<commit_message>
fix: clarify income draw capacity
- Rename income target to selected annual income draw
- Add max available annual income to inputs and engine output labels
- Update v2 spec, tests, and generated workbook
</commit_message>
<xml_diff>
--- a/btc_leveraged_model_v2.xlsx
+++ b/btc_leveraged_model_v2.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -790,11 +790,11 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Annual Income Target</t>
+          <t>Max Available Annual Income (Year 1)</t>
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>50000</v>
+        <v>42000</v>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
@@ -803,45 +803,65 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Borrow-funded income target</t>
+          <t>Calculated from BTC collateral, LTV ceiling, and liquidation buffer</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Income LTV Ceiling</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="n">
-        <v>0.35</v>
+          <t>Selected Annual Income Draw</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>50000</v>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Safe debt ceiling</t>
+          <t>User-selected draw; capped by max available annual income</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>Income LTV Ceiling</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Safe debt ceiling</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>Setup Collateral BTC</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n">
+      <c r="B20" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>Income keeps BTC constant</t>
         </is>
@@ -2037,7 +2057,7 @@
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
@@ -2094,12 +2114,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Requested Income</t>
+          <t>Selected Income Draw</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Available Borrowing Capacity</t>
+          <t>Max Available Annual Income</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -3252,7 +3272,7 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Income requested year 1</t>
+          <t>Income selected draw year 1</t>
         </is>
       </c>
       <c r="B13" s="11" t="n">

</xml_diff>

<commit_message>
fix: link price projection to inputs
- Add Annual BTC Price Growth input for editable price paths
- Make Price Projection BTC Price formulas reference Inputs
- Link engine BTC Price columns to the Price Projection tab
- Add regression coverage for the formula links
</commit_message>
<xml_diff>
--- a/btc_leveraged_model_v2.xlsx
+++ b/btc_leveraged_model_v2.xlsx
@@ -23,8 +23,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.00000000"/>
-    <numFmt numFmtId="165" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.00000000"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -138,22 +138,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -574,113 +574,113 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Starting BTC</t>
+          <t>Current BTC Price</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>2</v>
+        <v>60000</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>BTC</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Collateral used by both engines</t>
+          <t>Year 0 price; feeds Price Projection</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Current BTC Price</t>
+          <t>Annual BTC Price Growth</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>60000</v>
+        <v>0</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>%</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Year 0 price</t>
+          <t>Editable flat/default projection growth rate</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Borrow APR</t>
+          <t>Starting BTC</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>0.1</v>
+        <v>2</v>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Interest accrues on start-of-row debt</t>
+          <t>Collateral used by both engines</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Interest Treatment</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>capitalized</t>
-        </is>
+          <t>Borrow APR</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>0.1</v>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>choice</t>
+          <t>%</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>capitalized or paid externally</t>
+          <t>Interest accrues on start-of-row debt</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Margin Call LTV</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="n">
-        <v>0.7</v>
+          <t>Interest Treatment</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>capitalized</t>
+        </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>choice</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Risk threshold</t>
+          <t>capitalized or paid externally</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Liquidation LTV</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="n">
-        <v>0.75</v>
+          <t>Margin Call LTV</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>0.7</v>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
@@ -696,58 +696,58 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>Liquidation LTV</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Risk threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
           <t>Minimum Liquidation Buffer</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B12" s="8" t="n">
         <v>0.5</v>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>Required price-drop buffer</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Accumulation</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Target Effective LTV</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>Recursive setup/top-up target</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Max Effective LTV</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="n">
-        <v>0.35</v>
+          <t>Target Effective LTV</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n">
+        <v>0.25</v>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
@@ -756,65 +756,65 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Hard cap</t>
+          <t>Recursive setup/top-up target</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
+          <t>Max Effective LTV</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Hard cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
           <t>Setup Collateral BTC</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B16" s="9" t="n">
         <v>2.666666666666667</v>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>Computed audit output</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Income</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Max Available Annual Income (Year 1)</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="n">
-        <v>42000</v>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>Calculated from BTC collateral, LTV ceiling, and liquidation buffer</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Selected Annual Income Draw</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="n">
-        <v>50000</v>
+          <t>Max Available Annual Income (Year 1)</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>42000</v>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
@@ -823,45 +823,65 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>User-selected draw; capped by max available annual income</t>
+          <t>Calculated from BTC collateral, LTV ceiling, and liquidation buffer</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Income LTV Ceiling</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="n">
-        <v>0.35</v>
+          <t>Selected Annual Income Draw</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>50000</v>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Safe debt ceiling</t>
+          <t>User-selected draw; capped by max available annual income</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
+          <t>Income LTV Ceiling</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Safe debt ceiling</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
           <t>Setup Collateral BTC</t>
         </is>
       </c>
-      <c r="B20" s="5" t="n">
+      <c r="B21" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>Income keeps BTC constant</t>
         </is>
@@ -869,9 +889,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A17:D17"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A13:D13"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -888,8 +908,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -931,12 +951,13 @@
       <c r="A4" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="B4" s="11" t="n">
-        <v>60000</v>
+      <c r="B4" s="11">
+        <f>'Inputs'!$B$5</f>
+        <v/>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>Editable formula projection</t>
         </is>
       </c>
       <c r="D4" s="12" t="n">
@@ -947,160 +968,180 @@
       <c r="A5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="11" t="n">
-        <v>60000</v>
+      <c r="B5" s="11">
+        <f>B4*(1+'Inputs'!$B$6)</f>
+        <v/>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="n">
-        <v>0</v>
+          <t>Editable formula projection</t>
+        </is>
+      </c>
+      <c r="D5" s="12">
+        <f>B5/B4-1</f>
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="11" t="n">
-        <v>60000</v>
+      <c r="B6" s="11">
+        <f>B5*(1+'Inputs'!$B$6)</f>
+        <v/>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="n">
-        <v>0</v>
+          <t>Editable formula projection</t>
+        </is>
+      </c>
+      <c r="D6" s="12">
+        <f>B6/B5-1</f>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="11" t="n">
-        <v>60000</v>
+      <c r="B7" s="11">
+        <f>B6*(1+'Inputs'!$B$6)</f>
+        <v/>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="n">
-        <v>0</v>
+          <t>Editable formula projection</t>
+        </is>
+      </c>
+      <c r="D7" s="12">
+        <f>B7/B6-1</f>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="11" t="n">
-        <v>60000</v>
+      <c r="B8" s="11">
+        <f>B7*(1+'Inputs'!$B$6)</f>
+        <v/>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="n">
-        <v>0</v>
+          <t>Editable formula projection</t>
+        </is>
+      </c>
+      <c r="D8" s="12">
+        <f>B8/B7-1</f>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="11" t="n">
-        <v>60000</v>
+      <c r="B9" s="11">
+        <f>B8*(1+'Inputs'!$B$6)</f>
+        <v/>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="n">
-        <v>0</v>
+          <t>Editable formula projection</t>
+        </is>
+      </c>
+      <c r="D9" s="12">
+        <f>B9/B8-1</f>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="11" t="n">
-        <v>60000</v>
+      <c r="B10" s="11">
+        <f>B9*(1+'Inputs'!$B$6)</f>
+        <v/>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="n">
-        <v>0</v>
+          <t>Editable formula projection</t>
+        </is>
+      </c>
+      <c r="D10" s="12">
+        <f>B10/B9-1</f>
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="11" t="n">
-        <v>60000</v>
+      <c r="B11" s="11">
+        <f>B10*(1+'Inputs'!$B$6)</f>
+        <v/>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="n">
-        <v>0</v>
+          <t>Editable formula projection</t>
+        </is>
+      </c>
+      <c r="D11" s="12">
+        <f>B11/B10-1</f>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="11" t="n">
-        <v>60000</v>
+      <c r="B12" s="11">
+        <f>B11*(1+'Inputs'!$B$6)</f>
+        <v/>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="n">
-        <v>0</v>
+          <t>Editable formula projection</t>
+        </is>
+      </c>
+      <c r="D12" s="12">
+        <f>B12/B11-1</f>
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="11" t="n">
-        <v>60000</v>
+      <c r="B13" s="11">
+        <f>B12*(1+'Inputs'!$B$6)</f>
+        <v/>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="D13" s="12" t="n">
-        <v>0</v>
+          <t>Editable formula projection</t>
+        </is>
+      </c>
+      <c r="D13" s="12">
+        <f>B13/B12-1</f>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="11" t="n">
-        <v>60000</v>
+      <c r="B14" s="11">
+        <f>B13*(1+'Inputs'!$B$6)</f>
+        <v/>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="n">
-        <v>0</v>
+          <t>Editable formula projection</t>
+        </is>
+      </c>
+      <c r="D14" s="12">
+        <f>B14/B13-1</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -1121,7 +1162,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -1268,8 +1309,9 @@
       <c r="A4" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="B4" s="11" t="n">
-        <v>60000</v>
+      <c r="B4" s="11">
+        <f>'Price Projection'!B4</f>
+        <v/>
       </c>
       <c r="C4" s="13" t="n">
         <v>2</v>
@@ -1338,8 +1380,9 @@
       <c r="A5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="11" t="n">
-        <v>60000</v>
+      <c r="B5" s="11">
+        <f>'Price Projection'!B5</f>
+        <v/>
       </c>
       <c r="C5" s="13" t="n">
         <v>2.666666666666667</v>
@@ -1408,8 +1451,9 @@
       <c r="A6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="11" t="n">
-        <v>60000</v>
+      <c r="B6" s="11">
+        <f>'Price Projection'!B6</f>
+        <v/>
       </c>
       <c r="C6" s="13" t="n">
         <v>2.666666666666667</v>
@@ -1478,8 +1522,9 @@
       <c r="A7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="11" t="n">
-        <v>60000</v>
+      <c r="B7" s="11">
+        <f>'Price Projection'!B7</f>
+        <v/>
       </c>
       <c r="C7" s="13" t="n">
         <v>2.666666666666667</v>
@@ -1548,8 +1593,9 @@
       <c r="A8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="11" t="n">
-        <v>60000</v>
+      <c r="B8" s="11">
+        <f>'Price Projection'!B8</f>
+        <v/>
       </c>
       <c r="C8" s="13" t="n">
         <v>2.666666666666667</v>
@@ -1618,8 +1664,9 @@
       <c r="A9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="11" t="n">
-        <v>60000</v>
+      <c r="B9" s="11">
+        <f>'Price Projection'!B9</f>
+        <v/>
       </c>
       <c r="C9" s="13" t="n">
         <v>2.666666666666667</v>
@@ -1688,8 +1735,9 @@
       <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="11" t="n">
-        <v>60000</v>
+      <c r="B10" s="11">
+        <f>'Price Projection'!B10</f>
+        <v/>
       </c>
       <c r="C10" s="13" t="n">
         <v>2.666666666666667</v>
@@ -1758,8 +1806,9 @@
       <c r="A11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="11" t="n">
-        <v>60000</v>
+      <c r="B11" s="11">
+        <f>'Price Projection'!B11</f>
+        <v/>
       </c>
       <c r="C11" s="13" t="n">
         <v>2.666666666666667</v>
@@ -1828,8 +1877,9 @@
       <c r="A12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="11" t="n">
-        <v>60000</v>
+      <c r="B12" s="11">
+        <f>'Price Projection'!B12</f>
+        <v/>
       </c>
       <c r="C12" s="13" t="n">
         <v>2.666666666666667</v>
@@ -1898,8 +1948,9 @@
       <c r="A13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="11" t="n">
-        <v>60000</v>
+      <c r="B13" s="11">
+        <f>'Price Projection'!B13</f>
+        <v/>
       </c>
       <c r="C13" s="13" t="n">
         <v>2.666666666666667</v>
@@ -1968,8 +2019,9 @@
       <c r="A14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="11" t="n">
-        <v>60000</v>
+      <c r="B14" s="11">
+        <f>'Price Projection'!B14</f>
+        <v/>
       </c>
       <c r="C14" s="13" t="n">
         <v>2.666666666666667</v>
@@ -2052,7 +2104,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -2187,8 +2239,9 @@
       <c r="A4" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="B4" s="11" t="n">
-        <v>60000</v>
+      <c r="B4" s="11">
+        <f>'Price Projection'!B4</f>
+        <v/>
       </c>
       <c r="C4" s="13" t="n">
         <v>2</v>
@@ -2251,8 +2304,9 @@
       <c r="A5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="11" t="n">
-        <v>60000</v>
+      <c r="B5" s="11">
+        <f>'Price Projection'!B5</f>
+        <v/>
       </c>
       <c r="C5" s="13" t="n">
         <v>2</v>
@@ -2315,8 +2369,9 @@
       <c r="A6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="11" t="n">
-        <v>60000</v>
+      <c r="B6" s="11">
+        <f>'Price Projection'!B6</f>
+        <v/>
       </c>
       <c r="C6" s="13" t="n">
         <v>2</v>
@@ -2379,8 +2434,9 @@
       <c r="A7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="11" t="n">
-        <v>60000</v>
+      <c r="B7" s="11">
+        <f>'Price Projection'!B7</f>
+        <v/>
       </c>
       <c r="C7" s="13" t="n">
         <v>2</v>
@@ -2443,8 +2499,9 @@
       <c r="A8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="11" t="n">
-        <v>60000</v>
+      <c r="B8" s="11">
+        <f>'Price Projection'!B8</f>
+        <v/>
       </c>
       <c r="C8" s="13" t="n">
         <v>2</v>
@@ -2507,8 +2564,9 @@
       <c r="A9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="11" t="n">
-        <v>60000</v>
+      <c r="B9" s="11">
+        <f>'Price Projection'!B9</f>
+        <v/>
       </c>
       <c r="C9" s="13" t="n">
         <v>2</v>
@@ -2571,8 +2629,9 @@
       <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="11" t="n">
-        <v>60000</v>
+      <c r="B10" s="11">
+        <f>'Price Projection'!B10</f>
+        <v/>
       </c>
       <c r="C10" s="13" t="n">
         <v>2</v>
@@ -2635,8 +2694,9 @@
       <c r="A11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="11" t="n">
-        <v>60000</v>
+      <c r="B11" s="11">
+        <f>'Price Projection'!B11</f>
+        <v/>
       </c>
       <c r="C11" s="13" t="n">
         <v>2</v>
@@ -2699,8 +2759,9 @@
       <c r="A12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="11" t="n">
-        <v>60000</v>
+      <c r="B12" s="11">
+        <f>'Price Projection'!B12</f>
+        <v/>
       </c>
       <c r="C12" s="13" t="n">
         <v>2</v>
@@ -2763,8 +2824,9 @@
       <c r="A13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="11" t="n">
-        <v>60000</v>
+      <c r="B13" s="11">
+        <f>'Price Projection'!B13</f>
+        <v/>
       </c>
       <c r="C13" s="13" t="n">
         <v>2</v>
@@ -2827,8 +2889,9 @@
       <c r="A14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="11" t="n">
-        <v>60000</v>
+      <c r="B14" s="11">
+        <f>'Price Projection'!B14</f>
+        <v/>
       </c>
       <c r="C14" s="13" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
feat: make v2 workbook formula-native
- Convert accumulation, income, risk, and summary tabs to Excel formulas
- Keep price projection driven by editable Inputs values
- Add Warning LTV input and recalc-on-open workbook settings
- Add formula regression assertions for key workbook surfaces
</commit_message>
<xml_diff>
--- a/btc_leveraged_model_v2.xlsx
+++ b/btc_leveraged_model_v2.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Audit Examples" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -521,11 +521,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -786,8 +786,9 @@
           <t>Setup Collateral BTC</t>
         </is>
       </c>
-      <c r="B16" s="9" t="n">
-        <v>2.666666666666667</v>
+      <c r="B16" s="9">
+        <f>$B$7/(1-MIN($B$14,$B$15,$B$11*(1-$B$12)))</f>
+        <v/>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
@@ -796,7 +797,7 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Computed audit output</t>
+          <t>Formula output from starting BTC and effective LTV cap</t>
         </is>
       </c>
     </row>
@@ -813,8 +814,9 @@
           <t>Max Available Annual Income (Year 1)</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
-        <v>42000</v>
+      <c r="B18" s="5">
+        <f>MAX(0,$B$7*'Price Projection'!B5*MIN($B$20,$B$11*(1-$B$12)))</f>
+        <v/>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
@@ -823,7 +825,7 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Calculated from BTC collateral, LTV ceiling, and liquidation buffer</t>
+          <t>Formula output from BTC collateral, LTV ceiling, and liquidation buffer</t>
         </is>
       </c>
     </row>
@@ -873,8 +875,9 @@
           <t>Setup Collateral BTC</t>
         </is>
       </c>
-      <c r="B21" s="9" t="n">
-        <v>2</v>
+      <c r="B21" s="9">
+        <f>$B$7</f>
+        <v/>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
@@ -887,12 +890,40 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Advanced Risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Warning LTV</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Status changes to WARNING at or above this LTV</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A22:D22"/>
     <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A1:H1"/>
     <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1164,25 +1195,25 @@
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="21" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
     <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
-    <col width="21" customWidth="1" min="21" max="21"/>
-    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="28" customWidth="1" min="19" max="19"/>
+    <col width="28" customWidth="1" min="20" max="20"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
+    <col width="28" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1313,8 +1344,9 @@
         <f>'Price Projection'!B4</f>
         <v/>
       </c>
-      <c r="C4" s="13" t="n">
-        <v>2</v>
+      <c r="C4" s="13">
+        <f>'Inputs'!$B$7</f>
+        <v/>
       </c>
       <c r="D4" s="11" t="n">
         <v>0</v>
@@ -1322,58 +1354,73 @@
       <c r="E4" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="11" t="n">
-        <v>40000</v>
-      </c>
-      <c r="I4" s="13" t="n">
-        <v>0.6666666666666665</v>
-      </c>
-      <c r="J4" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="K4" s="11" t="n">
-        <v>40000</v>
-      </c>
-      <c r="L4" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="M4" s="13" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="N4" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="O4" s="13" t="n">
-        <v>0.6666666666666665</v>
-      </c>
-      <c r="P4" s="11" t="n">
-        <v>120000</v>
-      </c>
-      <c r="Q4" s="12" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="R4" s="6" t="n">
-        <v>1.333333333333333</v>
-      </c>
-      <c r="S4" s="11" t="n">
-        <v>21428.57142857143</v>
-      </c>
-      <c r="T4" s="11" t="n">
-        <v>20000</v>
-      </c>
-      <c r="U4" s="12" t="n">
-        <v>0.6666666666666667</v>
-      </c>
-      <c r="V4" s="6" t="inlineStr">
-        <is>
-          <t>SAFE</t>
-        </is>
+      <c r="F4" s="11">
+        <f>D4+E4</f>
+        <v/>
+      </c>
+      <c r="G4" s="12">
+        <f>IF(C4*B4=0,0,F4/(C4*B4))</f>
+        <v/>
+      </c>
+      <c r="H4" s="11">
+        <f>MAX(0,(MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12))*C4*B4-F4)/(1-MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12))))</f>
+        <v/>
+      </c>
+      <c r="I4" s="13">
+        <f>H4/B4</f>
+        <v/>
+      </c>
+      <c r="J4" s="13">
+        <f>C4+I4</f>
+        <v/>
+      </c>
+      <c r="K4" s="11">
+        <f>F4+H4</f>
+        <v/>
+      </c>
+      <c r="L4" s="13">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="M4" s="13">
+        <f>K4/B4</f>
+        <v/>
+      </c>
+      <c r="N4" s="13">
+        <f>L4-M4</f>
+        <v/>
+      </c>
+      <c r="O4" s="13">
+        <f>L4-'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="P4" s="11">
+        <f>L4*B4-K4</f>
+        <v/>
+      </c>
+      <c r="Q4" s="12">
+        <f>IF(J4*B4=0,0,K4/(J4*B4))</f>
+        <v/>
+      </c>
+      <c r="R4" s="6">
+        <f>L4/'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="S4" s="11">
+        <f>IF(K4=0,0,K4/(J4*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="T4" s="11">
+        <f>IF(K4=0,0,K4/(J4*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="U4" s="12">
+        <f>IF(T4&lt;=0,0,1-T4/B4)</f>
+        <v/>
+      </c>
+      <c r="V4" s="6">
+        <f>IF(Q4=0,"SAFE",IF(Q4&gt;='Inputs'!$B$11,"LIQUIDATED",IF(Q4&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(Q4&gt;='Inputs'!$B$23,U4&lt;'Inputs'!$B$12),"WARNING","SAFE"))))</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -1384,67 +1431,85 @@
         <f>'Price Projection'!B5</f>
         <v/>
       </c>
-      <c r="C5" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="D5" s="11" t="n">
-        <v>40000</v>
-      </c>
-      <c r="E5" s="11" t="n">
-        <v>4000</v>
-      </c>
-      <c r="F5" s="11" t="n">
-        <v>44000</v>
-      </c>
-      <c r="G5" s="12" t="n">
-        <v>0.275</v>
-      </c>
-      <c r="H5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="K5" s="11" t="n">
-        <v>44000</v>
-      </c>
-      <c r="L5" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="M5" s="13" t="n">
-        <v>0.7333333333333333</v>
-      </c>
-      <c r="N5" s="13" t="n">
-        <v>1.933333333333333</v>
-      </c>
-      <c r="O5" s="13" t="n">
-        <v>0.6666666666666665</v>
-      </c>
-      <c r="P5" s="11" t="n">
-        <v>116000</v>
-      </c>
-      <c r="Q5" s="12" t="n">
-        <v>0.275</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>1.333333333333333</v>
-      </c>
-      <c r="S5" s="11" t="n">
-        <v>23571.42857142857</v>
-      </c>
-      <c r="T5" s="11" t="n">
-        <v>22000</v>
-      </c>
-      <c r="U5" s="12" t="n">
-        <v>0.6333333333333333</v>
-      </c>
-      <c r="V5" s="6" t="inlineStr">
-        <is>
-          <t>SAFE</t>
-        </is>
+      <c r="C5" s="13">
+        <f>J4</f>
+        <v/>
+      </c>
+      <c r="D5" s="11">
+        <f>K4</f>
+        <v/>
+      </c>
+      <c r="E5" s="11">
+        <f>D5*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F5" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D5+E5,D5)</f>
+        <v/>
+      </c>
+      <c r="G5" s="12">
+        <f>IF(C5*B5=0,0,F5/(C5*B5))</f>
+        <v/>
+      </c>
+      <c r="H5" s="11">
+        <f>IF(G5&gt;='Inputs'!$B$10,0,MAX(0,(MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12))*C5*B5-F5)/(1-MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12)))))</f>
+        <v/>
+      </c>
+      <c r="I5" s="13">
+        <f>H5/B5</f>
+        <v/>
+      </c>
+      <c r="J5" s="13">
+        <f>C5+I5</f>
+        <v/>
+      </c>
+      <c r="K5" s="11">
+        <f>F5+H5</f>
+        <v/>
+      </c>
+      <c r="L5" s="13">
+        <f>J5</f>
+        <v/>
+      </c>
+      <c r="M5" s="13">
+        <f>K5/B5</f>
+        <v/>
+      </c>
+      <c r="N5" s="13">
+        <f>L5-M5</f>
+        <v/>
+      </c>
+      <c r="O5" s="13">
+        <f>L5-'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="P5" s="11">
+        <f>L5*B5-K5</f>
+        <v/>
+      </c>
+      <c r="Q5" s="12">
+        <f>IF(J5*B5=0,0,K5/(J5*B5))</f>
+        <v/>
+      </c>
+      <c r="R5" s="6">
+        <f>L5/'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="S5" s="11">
+        <f>IF(K5=0,0,K5/(J5*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="T5" s="11">
+        <f>IF(K5=0,0,K5/(J5*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="U5" s="12">
+        <f>IF(T5&lt;=0,0,1-T5/B5)</f>
+        <v/>
+      </c>
+      <c r="V5" s="6">
+        <f>IF(Q5=0,"SAFE",IF(Q5&gt;='Inputs'!$B$11,"LIQUIDATED",IF(Q5&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(Q5&gt;='Inputs'!$B$23,U5&lt;'Inputs'!$B$12),"WARNING","SAFE"))))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -1455,67 +1520,85 @@
         <f>'Price Projection'!B6</f>
         <v/>
       </c>
-      <c r="C6" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="D6" s="11" t="n">
-        <v>44000</v>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>4400</v>
-      </c>
-      <c r="F6" s="11" t="n">
-        <v>48400</v>
-      </c>
-      <c r="G6" s="12" t="n">
-        <v>0.3025</v>
-      </c>
-      <c r="H6" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="K6" s="11" t="n">
-        <v>48400</v>
-      </c>
-      <c r="L6" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="M6" s="13" t="n">
-        <v>0.8066666666666666</v>
-      </c>
-      <c r="N6" s="13" t="n">
-        <v>1.86</v>
-      </c>
-      <c r="O6" s="13" t="n">
-        <v>0.6666666666666665</v>
-      </c>
-      <c r="P6" s="11" t="n">
-        <v>111600</v>
-      </c>
-      <c r="Q6" s="12" t="n">
-        <v>0.3025</v>
-      </c>
-      <c r="R6" s="6" t="n">
-        <v>1.333333333333333</v>
-      </c>
-      <c r="S6" s="11" t="n">
-        <v>25928.57142857143</v>
-      </c>
-      <c r="T6" s="11" t="n">
-        <v>24200</v>
-      </c>
-      <c r="U6" s="12" t="n">
-        <v>0.5966666666666667</v>
-      </c>
-      <c r="V6" s="6" t="inlineStr">
-        <is>
-          <t>SAFE</t>
-        </is>
+      <c r="C6" s="13">
+        <f>J5</f>
+        <v/>
+      </c>
+      <c r="D6" s="11">
+        <f>K5</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>D6*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D6+E6,D6)</f>
+        <v/>
+      </c>
+      <c r="G6" s="12">
+        <f>IF(C6*B6=0,0,F6/(C6*B6))</f>
+        <v/>
+      </c>
+      <c r="H6" s="11">
+        <f>IF(G6&gt;='Inputs'!$B$10,0,MAX(0,(MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12))*C6*B6-F6)/(1-MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12)))))</f>
+        <v/>
+      </c>
+      <c r="I6" s="13">
+        <f>H6/B6</f>
+        <v/>
+      </c>
+      <c r="J6" s="13">
+        <f>C6+I6</f>
+        <v/>
+      </c>
+      <c r="K6" s="11">
+        <f>F6+H6</f>
+        <v/>
+      </c>
+      <c r="L6" s="13">
+        <f>J6</f>
+        <v/>
+      </c>
+      <c r="M6" s="13">
+        <f>K6/B6</f>
+        <v/>
+      </c>
+      <c r="N6" s="13">
+        <f>L6-M6</f>
+        <v/>
+      </c>
+      <c r="O6" s="13">
+        <f>L6-'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="P6" s="11">
+        <f>L6*B6-K6</f>
+        <v/>
+      </c>
+      <c r="Q6" s="12">
+        <f>IF(J6*B6=0,0,K6/(J6*B6))</f>
+        <v/>
+      </c>
+      <c r="R6" s="6">
+        <f>L6/'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="S6" s="11">
+        <f>IF(K6=0,0,K6/(J6*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="T6" s="11">
+        <f>IF(K6=0,0,K6/(J6*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="U6" s="12">
+        <f>IF(T6&lt;=0,0,1-T6/B6)</f>
+        <v/>
+      </c>
+      <c r="V6" s="6">
+        <f>IF(Q6=0,"SAFE",IF(Q6&gt;='Inputs'!$B$11,"LIQUIDATED",IF(Q6&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(Q6&gt;='Inputs'!$B$23,U6&lt;'Inputs'!$B$12),"WARNING","SAFE"))))</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -1526,67 +1609,85 @@
         <f>'Price Projection'!B7</f>
         <v/>
       </c>
-      <c r="C7" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="D7" s="11" t="n">
-        <v>48400</v>
-      </c>
-      <c r="E7" s="11" t="n">
-        <v>4840</v>
-      </c>
-      <c r="F7" s="11" t="n">
-        <v>53240</v>
-      </c>
-      <c r="G7" s="12" t="n">
-        <v>0.33275</v>
-      </c>
-      <c r="H7" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="K7" s="11" t="n">
-        <v>53240</v>
-      </c>
-      <c r="L7" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="M7" s="13" t="n">
-        <v>0.8873333333333333</v>
-      </c>
-      <c r="N7" s="13" t="n">
-        <v>1.779333333333333</v>
-      </c>
-      <c r="O7" s="13" t="n">
-        <v>0.6666666666666665</v>
-      </c>
-      <c r="P7" s="11" t="n">
-        <v>106760</v>
-      </c>
-      <c r="Q7" s="12" t="n">
-        <v>0.33275</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>1.333333333333333</v>
-      </c>
-      <c r="S7" s="11" t="n">
-        <v>28521.42857142858</v>
-      </c>
-      <c r="T7" s="11" t="n">
-        <v>26620</v>
-      </c>
-      <c r="U7" s="12" t="n">
-        <v>0.5563333333333333</v>
-      </c>
-      <c r="V7" s="6" t="inlineStr">
-        <is>
-          <t>SAFE</t>
-        </is>
+      <c r="C7" s="13">
+        <f>J6</f>
+        <v/>
+      </c>
+      <c r="D7" s="11">
+        <f>K6</f>
+        <v/>
+      </c>
+      <c r="E7" s="11">
+        <f>D7*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F7" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D7+E7,D7)</f>
+        <v/>
+      </c>
+      <c r="G7" s="12">
+        <f>IF(C7*B7=0,0,F7/(C7*B7))</f>
+        <v/>
+      </c>
+      <c r="H7" s="11">
+        <f>IF(G7&gt;='Inputs'!$B$10,0,MAX(0,(MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12))*C7*B7-F7)/(1-MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12)))))</f>
+        <v/>
+      </c>
+      <c r="I7" s="13">
+        <f>H7/B7</f>
+        <v/>
+      </c>
+      <c r="J7" s="13">
+        <f>C7+I7</f>
+        <v/>
+      </c>
+      <c r="K7" s="11">
+        <f>F7+H7</f>
+        <v/>
+      </c>
+      <c r="L7" s="13">
+        <f>J7</f>
+        <v/>
+      </c>
+      <c r="M7" s="13">
+        <f>K7/B7</f>
+        <v/>
+      </c>
+      <c r="N7" s="13">
+        <f>L7-M7</f>
+        <v/>
+      </c>
+      <c r="O7" s="13">
+        <f>L7-'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="P7" s="11">
+        <f>L7*B7-K7</f>
+        <v/>
+      </c>
+      <c r="Q7" s="12">
+        <f>IF(J7*B7=0,0,K7/(J7*B7))</f>
+        <v/>
+      </c>
+      <c r="R7" s="6">
+        <f>L7/'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="S7" s="11">
+        <f>IF(K7=0,0,K7/(J7*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="T7" s="11">
+        <f>IF(K7=0,0,K7/(J7*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="U7" s="12">
+        <f>IF(T7&lt;=0,0,1-T7/B7)</f>
+        <v/>
+      </c>
+      <c r="V7" s="6">
+        <f>IF(Q7=0,"SAFE",IF(Q7&gt;='Inputs'!$B$11,"LIQUIDATED",IF(Q7&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(Q7&gt;='Inputs'!$B$23,U7&lt;'Inputs'!$B$12),"WARNING","SAFE"))))</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -1597,67 +1698,85 @@
         <f>'Price Projection'!B8</f>
         <v/>
       </c>
-      <c r="C8" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="D8" s="11" t="n">
-        <v>53240</v>
-      </c>
-      <c r="E8" s="11" t="n">
-        <v>5324</v>
-      </c>
-      <c r="F8" s="11" t="n">
-        <v>58564</v>
-      </c>
-      <c r="G8" s="12" t="n">
-        <v>0.366025</v>
-      </c>
-      <c r="H8" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="K8" s="11" t="n">
-        <v>58564</v>
-      </c>
-      <c r="L8" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="M8" s="13" t="n">
-        <v>0.9760666666666666</v>
-      </c>
-      <c r="N8" s="13" t="n">
-        <v>1.6906</v>
-      </c>
-      <c r="O8" s="13" t="n">
-        <v>0.6666666666666665</v>
-      </c>
-      <c r="P8" s="11" t="n">
-        <v>101436</v>
-      </c>
-      <c r="Q8" s="12" t="n">
-        <v>0.366025</v>
-      </c>
-      <c r="R8" s="6" t="n">
-        <v>1.333333333333333</v>
-      </c>
-      <c r="S8" s="11" t="n">
-        <v>31373.57142857143</v>
-      </c>
-      <c r="T8" s="11" t="n">
-        <v>29282</v>
-      </c>
-      <c r="U8" s="12" t="n">
-        <v>0.5119666666666667</v>
-      </c>
-      <c r="V8" s="6" t="inlineStr">
-        <is>
-          <t>SAFE</t>
-        </is>
+      <c r="C8" s="13">
+        <f>J7</f>
+        <v/>
+      </c>
+      <c r="D8" s="11">
+        <f>K7</f>
+        <v/>
+      </c>
+      <c r="E8" s="11">
+        <f>D8*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F8" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D8+E8,D8)</f>
+        <v/>
+      </c>
+      <c r="G8" s="12">
+        <f>IF(C8*B8=0,0,F8/(C8*B8))</f>
+        <v/>
+      </c>
+      <c r="H8" s="11">
+        <f>IF(G8&gt;='Inputs'!$B$10,0,MAX(0,(MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12))*C8*B8-F8)/(1-MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12)))))</f>
+        <v/>
+      </c>
+      <c r="I8" s="13">
+        <f>H8/B8</f>
+        <v/>
+      </c>
+      <c r="J8" s="13">
+        <f>C8+I8</f>
+        <v/>
+      </c>
+      <c r="K8" s="11">
+        <f>F8+H8</f>
+        <v/>
+      </c>
+      <c r="L8" s="13">
+        <f>J8</f>
+        <v/>
+      </c>
+      <c r="M8" s="13">
+        <f>K8/B8</f>
+        <v/>
+      </c>
+      <c r="N8" s="13">
+        <f>L8-M8</f>
+        <v/>
+      </c>
+      <c r="O8" s="13">
+        <f>L8-'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="P8" s="11">
+        <f>L8*B8-K8</f>
+        <v/>
+      </c>
+      <c r="Q8" s="12">
+        <f>IF(J8*B8=0,0,K8/(J8*B8))</f>
+        <v/>
+      </c>
+      <c r="R8" s="6">
+        <f>L8/'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="S8" s="11">
+        <f>IF(K8=0,0,K8/(J8*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="T8" s="11">
+        <f>IF(K8=0,0,K8/(J8*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="U8" s="12">
+        <f>IF(T8&lt;=0,0,1-T8/B8)</f>
+        <v/>
+      </c>
+      <c r="V8" s="6">
+        <f>IF(Q8=0,"SAFE",IF(Q8&gt;='Inputs'!$B$11,"LIQUIDATED",IF(Q8&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(Q8&gt;='Inputs'!$B$23,U8&lt;'Inputs'!$B$12),"WARNING","SAFE"))))</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -1668,67 +1787,85 @@
         <f>'Price Projection'!B9</f>
         <v/>
       </c>
-      <c r="C9" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="D9" s="11" t="n">
-        <v>58564</v>
-      </c>
-      <c r="E9" s="11" t="n">
-        <v>5856.400000000001</v>
-      </c>
-      <c r="F9" s="11" t="n">
-        <v>64420.4</v>
-      </c>
-      <c r="G9" s="12" t="n">
-        <v>0.4026275</v>
-      </c>
-      <c r="H9" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="K9" s="11" t="n">
-        <v>64420.4</v>
-      </c>
-      <c r="L9" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="M9" s="13" t="n">
-        <v>1.073673333333333</v>
-      </c>
-      <c r="N9" s="13" t="n">
-        <v>1.592993333333333</v>
-      </c>
-      <c r="O9" s="13" t="n">
-        <v>0.6666666666666665</v>
-      </c>
-      <c r="P9" s="11" t="n">
-        <v>95579.60000000001</v>
-      </c>
-      <c r="Q9" s="12" t="n">
-        <v>0.4026275</v>
-      </c>
-      <c r="R9" s="6" t="n">
-        <v>1.333333333333333</v>
-      </c>
-      <c r="S9" s="11" t="n">
-        <v>34510.92857142857</v>
-      </c>
-      <c r="T9" s="11" t="n">
-        <v>32210.2</v>
-      </c>
-      <c r="U9" s="12" t="n">
-        <v>0.4631633333333334</v>
-      </c>
-      <c r="V9" s="6" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
+      <c r="C9" s="13">
+        <f>J8</f>
+        <v/>
+      </c>
+      <c r="D9" s="11">
+        <f>K8</f>
+        <v/>
+      </c>
+      <c r="E9" s="11">
+        <f>D9*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F9" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D9+E9,D9)</f>
+        <v/>
+      </c>
+      <c r="G9" s="12">
+        <f>IF(C9*B9=0,0,F9/(C9*B9))</f>
+        <v/>
+      </c>
+      <c r="H9" s="11">
+        <f>IF(G9&gt;='Inputs'!$B$10,0,MAX(0,(MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12))*C9*B9-F9)/(1-MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12)))))</f>
+        <v/>
+      </c>
+      <c r="I9" s="13">
+        <f>H9/B9</f>
+        <v/>
+      </c>
+      <c r="J9" s="13">
+        <f>C9+I9</f>
+        <v/>
+      </c>
+      <c r="K9" s="11">
+        <f>F9+H9</f>
+        <v/>
+      </c>
+      <c r="L9" s="13">
+        <f>J9</f>
+        <v/>
+      </c>
+      <c r="M9" s="13">
+        <f>K9/B9</f>
+        <v/>
+      </c>
+      <c r="N9" s="13">
+        <f>L9-M9</f>
+        <v/>
+      </c>
+      <c r="O9" s="13">
+        <f>L9-'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="P9" s="11">
+        <f>L9*B9-K9</f>
+        <v/>
+      </c>
+      <c r="Q9" s="12">
+        <f>IF(J9*B9=0,0,K9/(J9*B9))</f>
+        <v/>
+      </c>
+      <c r="R9" s="6">
+        <f>L9/'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="S9" s="11">
+        <f>IF(K9=0,0,K9/(J9*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="T9" s="11">
+        <f>IF(K9=0,0,K9/(J9*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="U9" s="12">
+        <f>IF(T9&lt;=0,0,1-T9/B9)</f>
+        <v/>
+      </c>
+      <c r="V9" s="6">
+        <f>IF(Q9=0,"SAFE",IF(Q9&gt;='Inputs'!$B$11,"LIQUIDATED",IF(Q9&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(Q9&gt;='Inputs'!$B$23,U9&lt;'Inputs'!$B$12),"WARNING","SAFE"))))</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -1739,67 +1876,85 @@
         <f>'Price Projection'!B10</f>
         <v/>
       </c>
-      <c r="C10" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="D10" s="11" t="n">
-        <v>64420.4</v>
-      </c>
-      <c r="E10" s="11" t="n">
-        <v>6442.040000000001</v>
-      </c>
-      <c r="F10" s="11" t="n">
-        <v>70862.44</v>
-      </c>
-      <c r="G10" s="12" t="n">
-        <v>0.44289025</v>
-      </c>
-      <c r="H10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="K10" s="11" t="n">
-        <v>70862.44</v>
-      </c>
-      <c r="L10" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="M10" s="13" t="n">
-        <v>1.181040666666667</v>
-      </c>
-      <c r="N10" s="13" t="n">
-        <v>1.485626</v>
-      </c>
-      <c r="O10" s="13" t="n">
-        <v>0.6666666666666665</v>
-      </c>
-      <c r="P10" s="11" t="n">
-        <v>89137.56</v>
-      </c>
-      <c r="Q10" s="12" t="n">
-        <v>0.44289025</v>
-      </c>
-      <c r="R10" s="6" t="n">
-        <v>1.333333333333333</v>
-      </c>
-      <c r="S10" s="11" t="n">
-        <v>37962.02142857143</v>
-      </c>
-      <c r="T10" s="11" t="n">
-        <v>35431.22</v>
-      </c>
-      <c r="U10" s="12" t="n">
-        <v>0.4094796666666667</v>
-      </c>
-      <c r="V10" s="6" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
+      <c r="C10" s="13">
+        <f>J9</f>
+        <v/>
+      </c>
+      <c r="D10" s="11">
+        <f>K9</f>
+        <v/>
+      </c>
+      <c r="E10" s="11">
+        <f>D10*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F10" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D10+E10,D10)</f>
+        <v/>
+      </c>
+      <c r="G10" s="12">
+        <f>IF(C10*B10=0,0,F10/(C10*B10))</f>
+        <v/>
+      </c>
+      <c r="H10" s="11">
+        <f>IF(G10&gt;='Inputs'!$B$10,0,MAX(0,(MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12))*C10*B10-F10)/(1-MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12)))))</f>
+        <v/>
+      </c>
+      <c r="I10" s="13">
+        <f>H10/B10</f>
+        <v/>
+      </c>
+      <c r="J10" s="13">
+        <f>C10+I10</f>
+        <v/>
+      </c>
+      <c r="K10" s="11">
+        <f>F10+H10</f>
+        <v/>
+      </c>
+      <c r="L10" s="13">
+        <f>J10</f>
+        <v/>
+      </c>
+      <c r="M10" s="13">
+        <f>K10/B10</f>
+        <v/>
+      </c>
+      <c r="N10" s="13">
+        <f>L10-M10</f>
+        <v/>
+      </c>
+      <c r="O10" s="13">
+        <f>L10-'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="P10" s="11">
+        <f>L10*B10-K10</f>
+        <v/>
+      </c>
+      <c r="Q10" s="12">
+        <f>IF(J10*B10=0,0,K10/(J10*B10))</f>
+        <v/>
+      </c>
+      <c r="R10" s="6">
+        <f>L10/'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="S10" s="11">
+        <f>IF(K10=0,0,K10/(J10*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="T10" s="11">
+        <f>IF(K10=0,0,K10/(J10*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="U10" s="12">
+        <f>IF(T10&lt;=0,0,1-T10/B10)</f>
+        <v/>
+      </c>
+      <c r="V10" s="6">
+        <f>IF(Q10=0,"SAFE",IF(Q10&gt;='Inputs'!$B$11,"LIQUIDATED",IF(Q10&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(Q10&gt;='Inputs'!$B$23,U10&lt;'Inputs'!$B$12),"WARNING","SAFE"))))</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -1810,67 +1965,85 @@
         <f>'Price Projection'!B11</f>
         <v/>
       </c>
-      <c r="C11" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="D11" s="11" t="n">
-        <v>70862.44</v>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>7086.244000000001</v>
-      </c>
-      <c r="F11" s="11" t="n">
-        <v>77948.68400000001</v>
-      </c>
-      <c r="G11" s="12" t="n">
-        <v>0.4871792750000001</v>
-      </c>
-      <c r="H11" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="K11" s="11" t="n">
-        <v>77948.68400000001</v>
-      </c>
-      <c r="L11" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="M11" s="13" t="n">
-        <v>1.299144733333333</v>
-      </c>
-      <c r="N11" s="13" t="n">
-        <v>1.367521933333333</v>
-      </c>
-      <c r="O11" s="13" t="n">
-        <v>0.6666666666666665</v>
-      </c>
-      <c r="P11" s="11" t="n">
-        <v>82051.31599999999</v>
-      </c>
-      <c r="Q11" s="12" t="n">
-        <v>0.4871792750000001</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>1.333333333333333</v>
-      </c>
-      <c r="S11" s="11" t="n">
-        <v>41758.22357142858</v>
-      </c>
-      <c r="T11" s="11" t="n">
-        <v>38974.342</v>
-      </c>
-      <c r="U11" s="12" t="n">
-        <v>0.3504276333333333</v>
-      </c>
-      <c r="V11" s="6" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
+      <c r="C11" s="13">
+        <f>J10</f>
+        <v/>
+      </c>
+      <c r="D11" s="11">
+        <f>K10</f>
+        <v/>
+      </c>
+      <c r="E11" s="11">
+        <f>D11*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F11" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D11+E11,D11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="12">
+        <f>IF(C11*B11=0,0,F11/(C11*B11))</f>
+        <v/>
+      </c>
+      <c r="H11" s="11">
+        <f>IF(G11&gt;='Inputs'!$B$10,0,MAX(0,(MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12))*C11*B11-F11)/(1-MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12)))))</f>
+        <v/>
+      </c>
+      <c r="I11" s="13">
+        <f>H11/B11</f>
+        <v/>
+      </c>
+      <c r="J11" s="13">
+        <f>C11+I11</f>
+        <v/>
+      </c>
+      <c r="K11" s="11">
+        <f>F11+H11</f>
+        <v/>
+      </c>
+      <c r="L11" s="13">
+        <f>J11</f>
+        <v/>
+      </c>
+      <c r="M11" s="13">
+        <f>K11/B11</f>
+        <v/>
+      </c>
+      <c r="N11" s="13">
+        <f>L11-M11</f>
+        <v/>
+      </c>
+      <c r="O11" s="13">
+        <f>L11-'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="P11" s="11">
+        <f>L11*B11-K11</f>
+        <v/>
+      </c>
+      <c r="Q11" s="12">
+        <f>IF(J11*B11=0,0,K11/(J11*B11))</f>
+        <v/>
+      </c>
+      <c r="R11" s="6">
+        <f>L11/'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="S11" s="11">
+        <f>IF(K11=0,0,K11/(J11*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="T11" s="11">
+        <f>IF(K11=0,0,K11/(J11*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="U11" s="12">
+        <f>IF(T11&lt;=0,0,1-T11/B11)</f>
+        <v/>
+      </c>
+      <c r="V11" s="6">
+        <f>IF(Q11=0,"SAFE",IF(Q11&gt;='Inputs'!$B$11,"LIQUIDATED",IF(Q11&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(Q11&gt;='Inputs'!$B$23,U11&lt;'Inputs'!$B$12),"WARNING","SAFE"))))</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -1881,67 +2054,85 @@
         <f>'Price Projection'!B12</f>
         <v/>
       </c>
-      <c r="C12" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="D12" s="11" t="n">
-        <v>77948.68400000001</v>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>7794.868400000001</v>
-      </c>
-      <c r="F12" s="11" t="n">
-        <v>85743.55240000002</v>
-      </c>
-      <c r="G12" s="12" t="n">
-        <v>0.5358972025000001</v>
-      </c>
-      <c r="H12" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="K12" s="11" t="n">
-        <v>85743.55240000002</v>
-      </c>
-      <c r="L12" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="M12" s="13" t="n">
-        <v>1.429059206666667</v>
-      </c>
-      <c r="N12" s="13" t="n">
-        <v>1.23760746</v>
-      </c>
-      <c r="O12" s="13" t="n">
-        <v>0.6666666666666665</v>
-      </c>
-      <c r="P12" s="11" t="n">
-        <v>74256.44759999998</v>
-      </c>
-      <c r="Q12" s="12" t="n">
-        <v>0.5358972025000001</v>
-      </c>
-      <c r="R12" s="6" t="n">
-        <v>1.333333333333333</v>
-      </c>
-      <c r="S12" s="11" t="n">
-        <v>45934.04592857144</v>
-      </c>
-      <c r="T12" s="11" t="n">
-        <v>42871.77620000001</v>
-      </c>
-      <c r="U12" s="12" t="n">
-        <v>0.2854703966666665</v>
-      </c>
-      <c r="V12" s="6" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
+      <c r="C12" s="13">
+        <f>J11</f>
+        <v/>
+      </c>
+      <c r="D12" s="11">
+        <f>K11</f>
+        <v/>
+      </c>
+      <c r="E12" s="11">
+        <f>D12*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F12" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D12+E12,D12)</f>
+        <v/>
+      </c>
+      <c r="G12" s="12">
+        <f>IF(C12*B12=0,0,F12/(C12*B12))</f>
+        <v/>
+      </c>
+      <c r="H12" s="11">
+        <f>IF(G12&gt;='Inputs'!$B$10,0,MAX(0,(MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12))*C12*B12-F12)/(1-MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12)))))</f>
+        <v/>
+      </c>
+      <c r="I12" s="13">
+        <f>H12/B12</f>
+        <v/>
+      </c>
+      <c r="J12" s="13">
+        <f>C12+I12</f>
+        <v/>
+      </c>
+      <c r="K12" s="11">
+        <f>F12+H12</f>
+        <v/>
+      </c>
+      <c r="L12" s="13">
+        <f>J12</f>
+        <v/>
+      </c>
+      <c r="M12" s="13">
+        <f>K12/B12</f>
+        <v/>
+      </c>
+      <c r="N12" s="13">
+        <f>L12-M12</f>
+        <v/>
+      </c>
+      <c r="O12" s="13">
+        <f>L12-'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="P12" s="11">
+        <f>L12*B12-K12</f>
+        <v/>
+      </c>
+      <c r="Q12" s="12">
+        <f>IF(J12*B12=0,0,K12/(J12*B12))</f>
+        <v/>
+      </c>
+      <c r="R12" s="6">
+        <f>L12/'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="S12" s="11">
+        <f>IF(K12=0,0,K12/(J12*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="T12" s="11">
+        <f>IF(K12=0,0,K12/(J12*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="U12" s="12">
+        <f>IF(T12&lt;=0,0,1-T12/B12)</f>
+        <v/>
+      </c>
+      <c r="V12" s="6">
+        <f>IF(Q12=0,"SAFE",IF(Q12&gt;='Inputs'!$B$11,"LIQUIDATED",IF(Q12&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(Q12&gt;='Inputs'!$B$23,U12&lt;'Inputs'!$B$12),"WARNING","SAFE"))))</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -1952,67 +2143,85 @@
         <f>'Price Projection'!B13</f>
         <v/>
       </c>
-      <c r="C13" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="D13" s="11" t="n">
-        <v>85743.55240000002</v>
-      </c>
-      <c r="E13" s="11" t="n">
-        <v>8574.355240000003</v>
-      </c>
-      <c r="F13" s="11" t="n">
-        <v>94317.90764000002</v>
-      </c>
-      <c r="G13" s="12" t="n">
-        <v>0.5894869227500001</v>
-      </c>
-      <c r="H13" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="K13" s="11" t="n">
-        <v>94317.90764000002</v>
-      </c>
-      <c r="L13" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="M13" s="13" t="n">
-        <v>1.571965127333334</v>
-      </c>
-      <c r="N13" s="13" t="n">
-        <v>1.094701539333333</v>
-      </c>
-      <c r="O13" s="13" t="n">
-        <v>0.6666666666666665</v>
-      </c>
-      <c r="P13" s="11" t="n">
-        <v>65682.09235999998</v>
-      </c>
-      <c r="Q13" s="12" t="n">
-        <v>0.5894869227500001</v>
-      </c>
-      <c r="R13" s="6" t="n">
-        <v>1.333333333333333</v>
-      </c>
-      <c r="S13" s="11" t="n">
-        <v>50527.45052142859</v>
-      </c>
-      <c r="T13" s="11" t="n">
-        <v>47158.95382000001</v>
-      </c>
-      <c r="U13" s="12" t="n">
-        <v>0.2140174363333331</v>
-      </c>
-      <c r="V13" s="6" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
+      <c r="C13" s="13">
+        <f>J12</f>
+        <v/>
+      </c>
+      <c r="D13" s="11">
+        <f>K12</f>
+        <v/>
+      </c>
+      <c r="E13" s="11">
+        <f>D13*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F13" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D13+E13,D13)</f>
+        <v/>
+      </c>
+      <c r="G13" s="12">
+        <f>IF(C13*B13=0,0,F13/(C13*B13))</f>
+        <v/>
+      </c>
+      <c r="H13" s="11">
+        <f>IF(G13&gt;='Inputs'!$B$10,0,MAX(0,(MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12))*C13*B13-F13)/(1-MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12)))))</f>
+        <v/>
+      </c>
+      <c r="I13" s="13">
+        <f>H13/B13</f>
+        <v/>
+      </c>
+      <c r="J13" s="13">
+        <f>C13+I13</f>
+        <v/>
+      </c>
+      <c r="K13" s="11">
+        <f>F13+H13</f>
+        <v/>
+      </c>
+      <c r="L13" s="13">
+        <f>J13</f>
+        <v/>
+      </c>
+      <c r="M13" s="13">
+        <f>K13/B13</f>
+        <v/>
+      </c>
+      <c r="N13" s="13">
+        <f>L13-M13</f>
+        <v/>
+      </c>
+      <c r="O13" s="13">
+        <f>L13-'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="P13" s="11">
+        <f>L13*B13-K13</f>
+        <v/>
+      </c>
+      <c r="Q13" s="12">
+        <f>IF(J13*B13=0,0,K13/(J13*B13))</f>
+        <v/>
+      </c>
+      <c r="R13" s="6">
+        <f>L13/'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="S13" s="11">
+        <f>IF(K13=0,0,K13/(J13*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="T13" s="11">
+        <f>IF(K13=0,0,K13/(J13*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="U13" s="12">
+        <f>IF(T13&lt;=0,0,1-T13/B13)</f>
+        <v/>
+      </c>
+      <c r="V13" s="6">
+        <f>IF(Q13=0,"SAFE",IF(Q13&gt;='Inputs'!$B$11,"LIQUIDATED",IF(Q13&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(Q13&gt;='Inputs'!$B$23,U13&lt;'Inputs'!$B$12),"WARNING","SAFE"))))</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -2023,67 +2232,85 @@
         <f>'Price Projection'!B14</f>
         <v/>
       </c>
-      <c r="C14" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="D14" s="11" t="n">
-        <v>94317.90764000002</v>
-      </c>
-      <c r="E14" s="11" t="n">
-        <v>9431.790764000003</v>
-      </c>
-      <c r="F14" s="11" t="n">
-        <v>103749.698404</v>
-      </c>
-      <c r="G14" s="12" t="n">
-        <v>0.6484356150250001</v>
-      </c>
-      <c r="H14" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="K14" s="11" t="n">
-        <v>103749.698404</v>
-      </c>
-      <c r="L14" s="13" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="M14" s="13" t="n">
-        <v>1.729161640066667</v>
-      </c>
-      <c r="N14" s="13" t="n">
-        <v>0.9375050265999993</v>
-      </c>
-      <c r="O14" s="13" t="n">
-        <v>0.6666666666666665</v>
-      </c>
-      <c r="P14" s="11" t="n">
-        <v>56250.30159599998</v>
-      </c>
-      <c r="Q14" s="12" t="n">
-        <v>0.6484356150250001</v>
-      </c>
-      <c r="R14" s="6" t="n">
-        <v>1.333333333333333</v>
-      </c>
-      <c r="S14" s="11" t="n">
-        <v>55580.19557357145</v>
-      </c>
-      <c r="T14" s="11" t="n">
-        <v>51874.84920200001</v>
-      </c>
-      <c r="U14" s="12" t="n">
-        <v>0.1354191799666664</v>
-      </c>
-      <c r="V14" s="6" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
+      <c r="C14" s="13">
+        <f>J13</f>
+        <v/>
+      </c>
+      <c r="D14" s="11">
+        <f>K13</f>
+        <v/>
+      </c>
+      <c r="E14" s="11">
+        <f>D14*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F14" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D14+E14,D14)</f>
+        <v/>
+      </c>
+      <c r="G14" s="12">
+        <f>IF(C14*B14=0,0,F14/(C14*B14))</f>
+        <v/>
+      </c>
+      <c r="H14" s="11">
+        <f>IF(G14&gt;='Inputs'!$B$10,0,MAX(0,(MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12))*C14*B14-F14)/(1-MIN('Inputs'!$B$14,'Inputs'!$B$15,'Inputs'!$B$11*(1-'Inputs'!$B$12)))))</f>
+        <v/>
+      </c>
+      <c r="I14" s="13">
+        <f>H14/B14</f>
+        <v/>
+      </c>
+      <c r="J14" s="13">
+        <f>C14+I14</f>
+        <v/>
+      </c>
+      <c r="K14" s="11">
+        <f>F14+H14</f>
+        <v/>
+      </c>
+      <c r="L14" s="13">
+        <f>J14</f>
+        <v/>
+      </c>
+      <c r="M14" s="13">
+        <f>K14/B14</f>
+        <v/>
+      </c>
+      <c r="N14" s="13">
+        <f>L14-M14</f>
+        <v/>
+      </c>
+      <c r="O14" s="13">
+        <f>L14-'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="P14" s="11">
+        <f>L14*B14-K14</f>
+        <v/>
+      </c>
+      <c r="Q14" s="12">
+        <f>IF(J14*B14=0,0,K14/(J14*B14))</f>
+        <v/>
+      </c>
+      <c r="R14" s="6">
+        <f>L14/'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="S14" s="11">
+        <f>IF(K14=0,0,K14/(J14*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="T14" s="11">
+        <f>IF(K14=0,0,K14/(J14*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="U14" s="12">
+        <f>IF(T14&lt;=0,0,1-T14/B14)</f>
+        <v/>
+      </c>
+      <c r="V14" s="6">
+        <f>IF(Q14=0,"SAFE",IF(Q14&gt;='Inputs'!$B$11,"LIQUIDATED",IF(Q14&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(Q14&gt;='Inputs'!$B$23,U14&lt;'Inputs'!$B$12),"WARNING","SAFE"))))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -2106,23 +2333,23 @@
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
-    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
-    <col width="21" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="24" customWidth="1" min="19" max="19"/>
-    <col width="23" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="28" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="28" customWidth="1" min="18" max="18"/>
+    <col width="25" customWidth="1" min="19" max="19"/>
+    <col width="28" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2243,8 +2470,9 @@
         <f>'Price Projection'!B4</f>
         <v/>
       </c>
-      <c r="C4" s="13" t="n">
-        <v>2</v>
+      <c r="C4" s="13">
+        <f>'Inputs'!$B$7</f>
+        <v/>
       </c>
       <c r="D4" s="11" t="n">
         <v>0</v>
@@ -2252,52 +2480,64 @@
       <c r="E4" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="11" t="n">
-        <v>0</v>
+      <c r="F4" s="11">
+        <f>D4+E4</f>
+        <v/>
       </c>
       <c r="G4" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="11" t="n">
-        <v>42000</v>
-      </c>
-      <c r="I4" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="O4" s="11" t="n">
-        <v>120000</v>
-      </c>
-      <c r="P4" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" s="6" t="inlineStr">
-        <is>
-          <t>SAFE</t>
-        </is>
+      <c r="H4" s="11">
+        <f>MAX(0,MIN(C4*B4*'Inputs'!$B$20,C4*B4*'Inputs'!$B$11*(1-'Inputs'!$B$12))-F4)</f>
+        <v/>
+      </c>
+      <c r="I4" s="11">
+        <f>IF(IF(C4*B4=0,0,F4/(C4*B4))&gt;='Inputs'!$B$10,0,MIN(G4,H4))</f>
+        <v/>
+      </c>
+      <c r="J4" s="11">
+        <f>G4-I4</f>
+        <v/>
+      </c>
+      <c r="K4" s="11">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="L4" s="11">
+        <f>F4+I4</f>
+        <v/>
+      </c>
+      <c r="M4" s="13">
+        <f>L4/B4</f>
+        <v/>
+      </c>
+      <c r="N4" s="13">
+        <f>C4-M4</f>
+        <v/>
+      </c>
+      <c r="O4" s="11">
+        <f>C4*B4-L4</f>
+        <v/>
+      </c>
+      <c r="P4" s="12">
+        <f>IF(C4*B4=0,0,L4/(C4*B4))</f>
+        <v/>
+      </c>
+      <c r="Q4" s="11">
+        <f>IF(L4=0,0,L4/(C4*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="R4" s="11">
+        <f>IF(L4=0,0,L4/(C4*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="S4" s="12">
+        <f>IF(R4&lt;=0,0,1-R4/B4)</f>
+        <v/>
+      </c>
+      <c r="T4" s="6">
+        <f>IF(P4&gt;='Inputs'!$B$11,"LIQUIDATED",IF(P4&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(P4&gt;='Inputs'!$B$23,S4&lt;'Inputs'!$B$12),"WARNING",IF(AND(G4&gt;0,I4=0),"FAILED",IF(I4&lt;G4,"CONSTRAINED","SAFE")))))</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -2308,61 +2548,77 @@
         <f>'Price Projection'!B5</f>
         <v/>
       </c>
-      <c r="C5" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="H5" s="11" t="n">
-        <v>42000</v>
-      </c>
-      <c r="I5" s="11" t="n">
-        <v>42000</v>
-      </c>
-      <c r="J5" s="11" t="n">
-        <v>8000</v>
-      </c>
-      <c r="K5" s="11" t="n">
-        <v>42000</v>
-      </c>
-      <c r="L5" s="11" t="n">
-        <v>42000</v>
-      </c>
-      <c r="M5" s="13" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="N5" s="13" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="O5" s="11" t="n">
-        <v>78000</v>
-      </c>
-      <c r="P5" s="12" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="Q5" s="11" t="n">
-        <v>30000</v>
-      </c>
-      <c r="R5" s="11" t="n">
-        <v>28000</v>
-      </c>
-      <c r="S5" s="12" t="n">
-        <v>0.5333333333333333</v>
-      </c>
-      <c r="T5" s="6" t="inlineStr">
-        <is>
-          <t>CONSTRAINED</t>
-        </is>
+      <c r="C5" s="13">
+        <f>'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="D5" s="11">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="E5" s="11">
+        <f>D5*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F5" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D5+E5,D5)</f>
+        <v/>
+      </c>
+      <c r="G5" s="11">
+        <f>'Inputs'!$B$19</f>
+        <v/>
+      </c>
+      <c r="H5" s="11">
+        <f>MAX(0,MIN(C5*B5*'Inputs'!$B$20,C5*B5*'Inputs'!$B$11*(1-'Inputs'!$B$12))-F5)</f>
+        <v/>
+      </c>
+      <c r="I5" s="11">
+        <f>IF(IF(C5*B5=0,0,F5/(C5*B5))&gt;='Inputs'!$B$10,0,MIN(G5,H5))</f>
+        <v/>
+      </c>
+      <c r="J5" s="11">
+        <f>G5-I5</f>
+        <v/>
+      </c>
+      <c r="K5" s="11">
+        <f>K4+I5</f>
+        <v/>
+      </c>
+      <c r="L5" s="11">
+        <f>F5+I5</f>
+        <v/>
+      </c>
+      <c r="M5" s="13">
+        <f>L5/B5</f>
+        <v/>
+      </c>
+      <c r="N5" s="13">
+        <f>C5-M5</f>
+        <v/>
+      </c>
+      <c r="O5" s="11">
+        <f>C5*B5-L5</f>
+        <v/>
+      </c>
+      <c r="P5" s="12">
+        <f>IF(C5*B5=0,0,L5/(C5*B5))</f>
+        <v/>
+      </c>
+      <c r="Q5" s="11">
+        <f>IF(L5=0,0,L5/(C5*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="R5" s="11">
+        <f>IF(L5=0,0,L5/(C5*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="S5" s="12">
+        <f>IF(R5&lt;=0,0,1-R5/B5)</f>
+        <v/>
+      </c>
+      <c r="T5" s="6">
+        <f>IF(P5&gt;='Inputs'!$B$11,"LIQUIDATED",IF(P5&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(P5&gt;='Inputs'!$B$23,S5&lt;'Inputs'!$B$12),"WARNING",IF(AND(G5&gt;0,I5=0),"FAILED",IF(I5&lt;G5,"CONSTRAINED","SAFE")))))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -2373,61 +2629,77 @@
         <f>'Price Projection'!B6</f>
         <v/>
       </c>
-      <c r="C6" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="11" t="n">
-        <v>42000</v>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>4200</v>
-      </c>
-      <c r="F6" s="11" t="n">
-        <v>46200</v>
-      </c>
-      <c r="G6" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="H6" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="K6" s="11" t="n">
-        <v>42000</v>
-      </c>
-      <c r="L6" s="11" t="n">
-        <v>46200</v>
-      </c>
-      <c r="M6" s="13" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="N6" s="13" t="n">
-        <v>1.23</v>
-      </c>
-      <c r="O6" s="11" t="n">
-        <v>73800</v>
-      </c>
-      <c r="P6" s="12" t="n">
-        <v>0.385</v>
-      </c>
-      <c r="Q6" s="11" t="n">
-        <v>33000</v>
-      </c>
-      <c r="R6" s="11" t="n">
-        <v>30800</v>
-      </c>
-      <c r="S6" s="12" t="n">
-        <v>0.4866666666666667</v>
-      </c>
-      <c r="T6" s="6" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
+      <c r="C6" s="13">
+        <f>'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="D6" s="11">
+        <f>L5</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>D6*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D6+E6,D6)</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
+        <f>'Inputs'!$B$19</f>
+        <v/>
+      </c>
+      <c r="H6" s="11">
+        <f>MAX(0,MIN(C6*B6*'Inputs'!$B$20,C6*B6*'Inputs'!$B$11*(1-'Inputs'!$B$12))-F6)</f>
+        <v/>
+      </c>
+      <c r="I6" s="11">
+        <f>IF(IF(C6*B6=0,0,F6/(C6*B6))&gt;='Inputs'!$B$10,0,MIN(G6,H6))</f>
+        <v/>
+      </c>
+      <c r="J6" s="11">
+        <f>G6-I6</f>
+        <v/>
+      </c>
+      <c r="K6" s="11">
+        <f>K5+I6</f>
+        <v/>
+      </c>
+      <c r="L6" s="11">
+        <f>F6+I6</f>
+        <v/>
+      </c>
+      <c r="M6" s="13">
+        <f>L6/B6</f>
+        <v/>
+      </c>
+      <c r="N6" s="13">
+        <f>C6-M6</f>
+        <v/>
+      </c>
+      <c r="O6" s="11">
+        <f>C6*B6-L6</f>
+        <v/>
+      </c>
+      <c r="P6" s="12">
+        <f>IF(C6*B6=0,0,L6/(C6*B6))</f>
+        <v/>
+      </c>
+      <c r="Q6" s="11">
+        <f>IF(L6=0,0,L6/(C6*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="R6" s="11">
+        <f>IF(L6=0,0,L6/(C6*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="S6" s="12">
+        <f>IF(R6&lt;=0,0,1-R6/B6)</f>
+        <v/>
+      </c>
+      <c r="T6" s="6">
+        <f>IF(P6&gt;='Inputs'!$B$11,"LIQUIDATED",IF(P6&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(P6&gt;='Inputs'!$B$23,S6&lt;'Inputs'!$B$12),"WARNING",IF(AND(G6&gt;0,I6=0),"FAILED",IF(I6&lt;G6,"CONSTRAINED","SAFE")))))</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -2438,61 +2710,77 @@
         <f>'Price Projection'!B7</f>
         <v/>
       </c>
-      <c r="C7" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="11" t="n">
-        <v>46200</v>
-      </c>
-      <c r="E7" s="11" t="n">
-        <v>4620</v>
-      </c>
-      <c r="F7" s="11" t="n">
-        <v>50820</v>
-      </c>
-      <c r="G7" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="H7" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="K7" s="11" t="n">
-        <v>42000</v>
-      </c>
-      <c r="L7" s="11" t="n">
-        <v>50820</v>
-      </c>
-      <c r="M7" s="13" t="n">
-        <v>0.847</v>
-      </c>
-      <c r="N7" s="13" t="n">
-        <v>1.153</v>
-      </c>
-      <c r="O7" s="11" t="n">
-        <v>69180</v>
-      </c>
-      <c r="P7" s="12" t="n">
-        <v>0.4235</v>
-      </c>
-      <c r="Q7" s="11" t="n">
-        <v>36300</v>
-      </c>
-      <c r="R7" s="11" t="n">
-        <v>33880</v>
-      </c>
-      <c r="S7" s="12" t="n">
-        <v>0.4353333333333333</v>
-      </c>
-      <c r="T7" s="6" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
+      <c r="C7" s="13">
+        <f>'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="D7" s="11">
+        <f>L6</f>
+        <v/>
+      </c>
+      <c r="E7" s="11">
+        <f>D7*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F7" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D7+E7,D7)</f>
+        <v/>
+      </c>
+      <c r="G7" s="11">
+        <f>'Inputs'!$B$19</f>
+        <v/>
+      </c>
+      <c r="H7" s="11">
+        <f>MAX(0,MIN(C7*B7*'Inputs'!$B$20,C7*B7*'Inputs'!$B$11*(1-'Inputs'!$B$12))-F7)</f>
+        <v/>
+      </c>
+      <c r="I7" s="11">
+        <f>IF(IF(C7*B7=0,0,F7/(C7*B7))&gt;='Inputs'!$B$10,0,MIN(G7,H7))</f>
+        <v/>
+      </c>
+      <c r="J7" s="11">
+        <f>G7-I7</f>
+        <v/>
+      </c>
+      <c r="K7" s="11">
+        <f>K6+I7</f>
+        <v/>
+      </c>
+      <c r="L7" s="11">
+        <f>F7+I7</f>
+        <v/>
+      </c>
+      <c r="M7" s="13">
+        <f>L7/B7</f>
+        <v/>
+      </c>
+      <c r="N7" s="13">
+        <f>C7-M7</f>
+        <v/>
+      </c>
+      <c r="O7" s="11">
+        <f>C7*B7-L7</f>
+        <v/>
+      </c>
+      <c r="P7" s="12">
+        <f>IF(C7*B7=0,0,L7/(C7*B7))</f>
+        <v/>
+      </c>
+      <c r="Q7" s="11">
+        <f>IF(L7=0,0,L7/(C7*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="R7" s="11">
+        <f>IF(L7=0,0,L7/(C7*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="S7" s="12">
+        <f>IF(R7&lt;=0,0,1-R7/B7)</f>
+        <v/>
+      </c>
+      <c r="T7" s="6">
+        <f>IF(P7&gt;='Inputs'!$B$11,"LIQUIDATED",IF(P7&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(P7&gt;='Inputs'!$B$23,S7&lt;'Inputs'!$B$12),"WARNING",IF(AND(G7&gt;0,I7=0),"FAILED",IF(I7&lt;G7,"CONSTRAINED","SAFE")))))</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -2503,61 +2791,77 @@
         <f>'Price Projection'!B8</f>
         <v/>
       </c>
-      <c r="C8" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" s="11" t="n">
-        <v>50820</v>
-      </c>
-      <c r="E8" s="11" t="n">
-        <v>5082</v>
-      </c>
-      <c r="F8" s="11" t="n">
-        <v>55902</v>
-      </c>
-      <c r="G8" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="H8" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="K8" s="11" t="n">
-        <v>42000</v>
-      </c>
-      <c r="L8" s="11" t="n">
-        <v>55902</v>
-      </c>
-      <c r="M8" s="13" t="n">
-        <v>0.9317</v>
-      </c>
-      <c r="N8" s="13" t="n">
-        <v>1.0683</v>
-      </c>
-      <c r="O8" s="11" t="n">
-        <v>64098</v>
-      </c>
-      <c r="P8" s="12" t="n">
-        <v>0.46585</v>
-      </c>
-      <c r="Q8" s="11" t="n">
-        <v>39930</v>
-      </c>
-      <c r="R8" s="11" t="n">
-        <v>37268</v>
-      </c>
-      <c r="S8" s="12" t="n">
-        <v>0.3788666666666667</v>
-      </c>
-      <c r="T8" s="6" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
+      <c r="C8" s="13">
+        <f>'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="D8" s="11">
+        <f>L7</f>
+        <v/>
+      </c>
+      <c r="E8" s="11">
+        <f>D8*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F8" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D8+E8,D8)</f>
+        <v/>
+      </c>
+      <c r="G8" s="11">
+        <f>'Inputs'!$B$19</f>
+        <v/>
+      </c>
+      <c r="H8" s="11">
+        <f>MAX(0,MIN(C8*B8*'Inputs'!$B$20,C8*B8*'Inputs'!$B$11*(1-'Inputs'!$B$12))-F8)</f>
+        <v/>
+      </c>
+      <c r="I8" s="11">
+        <f>IF(IF(C8*B8=0,0,F8/(C8*B8))&gt;='Inputs'!$B$10,0,MIN(G8,H8))</f>
+        <v/>
+      </c>
+      <c r="J8" s="11">
+        <f>G8-I8</f>
+        <v/>
+      </c>
+      <c r="K8" s="11">
+        <f>K7+I8</f>
+        <v/>
+      </c>
+      <c r="L8" s="11">
+        <f>F8+I8</f>
+        <v/>
+      </c>
+      <c r="M8" s="13">
+        <f>L8/B8</f>
+        <v/>
+      </c>
+      <c r="N8" s="13">
+        <f>C8-M8</f>
+        <v/>
+      </c>
+      <c r="O8" s="11">
+        <f>C8*B8-L8</f>
+        <v/>
+      </c>
+      <c r="P8" s="12">
+        <f>IF(C8*B8=0,0,L8/(C8*B8))</f>
+        <v/>
+      </c>
+      <c r="Q8" s="11">
+        <f>IF(L8=0,0,L8/(C8*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="R8" s="11">
+        <f>IF(L8=0,0,L8/(C8*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="S8" s="12">
+        <f>IF(R8&lt;=0,0,1-R8/B8)</f>
+        <v/>
+      </c>
+      <c r="T8" s="6">
+        <f>IF(P8&gt;='Inputs'!$B$11,"LIQUIDATED",IF(P8&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(P8&gt;='Inputs'!$B$23,S8&lt;'Inputs'!$B$12),"WARNING",IF(AND(G8&gt;0,I8=0),"FAILED",IF(I8&lt;G8,"CONSTRAINED","SAFE")))))</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -2568,61 +2872,77 @@
         <f>'Price Projection'!B9</f>
         <v/>
       </c>
-      <c r="C9" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D9" s="11" t="n">
-        <v>55902</v>
-      </c>
-      <c r="E9" s="11" t="n">
-        <v>5590.200000000001</v>
-      </c>
-      <c r="F9" s="11" t="n">
-        <v>61492.2</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="H9" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="K9" s="11" t="n">
-        <v>42000</v>
-      </c>
-      <c r="L9" s="11" t="n">
-        <v>61492.2</v>
-      </c>
-      <c r="M9" s="13" t="n">
-        <v>1.02487</v>
-      </c>
-      <c r="N9" s="13" t="n">
-        <v>0.9751300000000001</v>
-      </c>
-      <c r="O9" s="11" t="n">
-        <v>58507.8</v>
-      </c>
-      <c r="P9" s="12" t="n">
-        <v>0.512435</v>
-      </c>
-      <c r="Q9" s="11" t="n">
-        <v>43923</v>
-      </c>
-      <c r="R9" s="11" t="n">
-        <v>40994.8</v>
-      </c>
-      <c r="S9" s="12" t="n">
-        <v>0.3167533333333334</v>
-      </c>
-      <c r="T9" s="6" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
+      <c r="C9" s="13">
+        <f>'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="D9" s="11">
+        <f>L8</f>
+        <v/>
+      </c>
+      <c r="E9" s="11">
+        <f>D9*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F9" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D9+E9,D9)</f>
+        <v/>
+      </c>
+      <c r="G9" s="11">
+        <f>'Inputs'!$B$19</f>
+        <v/>
+      </c>
+      <c r="H9" s="11">
+        <f>MAX(0,MIN(C9*B9*'Inputs'!$B$20,C9*B9*'Inputs'!$B$11*(1-'Inputs'!$B$12))-F9)</f>
+        <v/>
+      </c>
+      <c r="I9" s="11">
+        <f>IF(IF(C9*B9=0,0,F9/(C9*B9))&gt;='Inputs'!$B$10,0,MIN(G9,H9))</f>
+        <v/>
+      </c>
+      <c r="J9" s="11">
+        <f>G9-I9</f>
+        <v/>
+      </c>
+      <c r="K9" s="11">
+        <f>K8+I9</f>
+        <v/>
+      </c>
+      <c r="L9" s="11">
+        <f>F9+I9</f>
+        <v/>
+      </c>
+      <c r="M9" s="13">
+        <f>L9/B9</f>
+        <v/>
+      </c>
+      <c r="N9" s="13">
+        <f>C9-M9</f>
+        <v/>
+      </c>
+      <c r="O9" s="11">
+        <f>C9*B9-L9</f>
+        <v/>
+      </c>
+      <c r="P9" s="12">
+        <f>IF(C9*B9=0,0,L9/(C9*B9))</f>
+        <v/>
+      </c>
+      <c r="Q9" s="11">
+        <f>IF(L9=0,0,L9/(C9*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="R9" s="11">
+        <f>IF(L9=0,0,L9/(C9*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="S9" s="12">
+        <f>IF(R9&lt;=0,0,1-R9/B9)</f>
+        <v/>
+      </c>
+      <c r="T9" s="6">
+        <f>IF(P9&gt;='Inputs'!$B$11,"LIQUIDATED",IF(P9&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(P9&gt;='Inputs'!$B$23,S9&lt;'Inputs'!$B$12),"WARNING",IF(AND(G9&gt;0,I9=0),"FAILED",IF(I9&lt;G9,"CONSTRAINED","SAFE")))))</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -2633,61 +2953,77 @@
         <f>'Price Projection'!B10</f>
         <v/>
       </c>
-      <c r="C10" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D10" s="11" t="n">
-        <v>61492.2</v>
-      </c>
-      <c r="E10" s="11" t="n">
-        <v>6149.22</v>
-      </c>
-      <c r="F10" s="11" t="n">
-        <v>67641.42</v>
-      </c>
-      <c r="G10" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="H10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="K10" s="11" t="n">
-        <v>42000</v>
-      </c>
-      <c r="L10" s="11" t="n">
-        <v>67641.42</v>
-      </c>
-      <c r="M10" s="13" t="n">
-        <v>1.127357</v>
-      </c>
-      <c r="N10" s="13" t="n">
-        <v>0.8726430000000001</v>
-      </c>
-      <c r="O10" s="11" t="n">
-        <v>52358.58</v>
-      </c>
-      <c r="P10" s="12" t="n">
-        <v>0.5636785</v>
-      </c>
-      <c r="Q10" s="11" t="n">
-        <v>48315.3</v>
-      </c>
-      <c r="R10" s="11" t="n">
-        <v>45094.28</v>
-      </c>
-      <c r="S10" s="12" t="n">
-        <v>0.2484286666666666</v>
-      </c>
-      <c r="T10" s="6" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
+      <c r="C10" s="13">
+        <f>'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="D10" s="11">
+        <f>L9</f>
+        <v/>
+      </c>
+      <c r="E10" s="11">
+        <f>D10*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F10" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D10+E10,D10)</f>
+        <v/>
+      </c>
+      <c r="G10" s="11">
+        <f>'Inputs'!$B$19</f>
+        <v/>
+      </c>
+      <c r="H10" s="11">
+        <f>MAX(0,MIN(C10*B10*'Inputs'!$B$20,C10*B10*'Inputs'!$B$11*(1-'Inputs'!$B$12))-F10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="11">
+        <f>IF(IF(C10*B10=0,0,F10/(C10*B10))&gt;='Inputs'!$B$10,0,MIN(G10,H10))</f>
+        <v/>
+      </c>
+      <c r="J10" s="11">
+        <f>G10-I10</f>
+        <v/>
+      </c>
+      <c r="K10" s="11">
+        <f>K9+I10</f>
+        <v/>
+      </c>
+      <c r="L10" s="11">
+        <f>F10+I10</f>
+        <v/>
+      </c>
+      <c r="M10" s="13">
+        <f>L10/B10</f>
+        <v/>
+      </c>
+      <c r="N10" s="13">
+        <f>C10-M10</f>
+        <v/>
+      </c>
+      <c r="O10" s="11">
+        <f>C10*B10-L10</f>
+        <v/>
+      </c>
+      <c r="P10" s="12">
+        <f>IF(C10*B10=0,0,L10/(C10*B10))</f>
+        <v/>
+      </c>
+      <c r="Q10" s="11">
+        <f>IF(L10=0,0,L10/(C10*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="R10" s="11">
+        <f>IF(L10=0,0,L10/(C10*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="S10" s="12">
+        <f>IF(R10&lt;=0,0,1-R10/B10)</f>
+        <v/>
+      </c>
+      <c r="T10" s="6">
+        <f>IF(P10&gt;='Inputs'!$B$11,"LIQUIDATED",IF(P10&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(P10&gt;='Inputs'!$B$23,S10&lt;'Inputs'!$B$12),"WARNING",IF(AND(G10&gt;0,I10=0),"FAILED",IF(I10&lt;G10,"CONSTRAINED","SAFE")))))</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -2698,61 +3034,77 @@
         <f>'Price Projection'!B11</f>
         <v/>
       </c>
-      <c r="C11" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" s="11" t="n">
-        <v>67641.42</v>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>6764.142</v>
-      </c>
-      <c r="F11" s="11" t="n">
-        <v>74405.56200000001</v>
-      </c>
-      <c r="G11" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="H11" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="K11" s="11" t="n">
-        <v>42000</v>
-      </c>
-      <c r="L11" s="11" t="n">
-        <v>74405.56200000001</v>
-      </c>
-      <c r="M11" s="13" t="n">
-        <v>1.2400927</v>
-      </c>
-      <c r="N11" s="13" t="n">
-        <v>0.7599072999999998</v>
-      </c>
-      <c r="O11" s="11" t="n">
-        <v>45594.43799999999</v>
-      </c>
-      <c r="P11" s="12" t="n">
-        <v>0.6200463500000001</v>
-      </c>
-      <c r="Q11" s="11" t="n">
-        <v>53146.83000000001</v>
-      </c>
-      <c r="R11" s="11" t="n">
-        <v>49603.70800000001</v>
-      </c>
-      <c r="S11" s="12" t="n">
-        <v>0.1732715333333332</v>
-      </c>
-      <c r="T11" s="6" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
+      <c r="C11" s="13">
+        <f>'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="D11" s="11">
+        <f>L10</f>
+        <v/>
+      </c>
+      <c r="E11" s="11">
+        <f>D11*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F11" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D11+E11,D11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="11">
+        <f>'Inputs'!$B$19</f>
+        <v/>
+      </c>
+      <c r="H11" s="11">
+        <f>MAX(0,MIN(C11*B11*'Inputs'!$B$20,C11*B11*'Inputs'!$B$11*(1-'Inputs'!$B$12))-F11)</f>
+        <v/>
+      </c>
+      <c r="I11" s="11">
+        <f>IF(IF(C11*B11=0,0,F11/(C11*B11))&gt;='Inputs'!$B$10,0,MIN(G11,H11))</f>
+        <v/>
+      </c>
+      <c r="J11" s="11">
+        <f>G11-I11</f>
+        <v/>
+      </c>
+      <c r="K11" s="11">
+        <f>K10+I11</f>
+        <v/>
+      </c>
+      <c r="L11" s="11">
+        <f>F11+I11</f>
+        <v/>
+      </c>
+      <c r="M11" s="13">
+        <f>L11/B11</f>
+        <v/>
+      </c>
+      <c r="N11" s="13">
+        <f>C11-M11</f>
+        <v/>
+      </c>
+      <c r="O11" s="11">
+        <f>C11*B11-L11</f>
+        <v/>
+      </c>
+      <c r="P11" s="12">
+        <f>IF(C11*B11=0,0,L11/(C11*B11))</f>
+        <v/>
+      </c>
+      <c r="Q11" s="11">
+        <f>IF(L11=0,0,L11/(C11*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="R11" s="11">
+        <f>IF(L11=0,0,L11/(C11*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="S11" s="12">
+        <f>IF(R11&lt;=0,0,1-R11/B11)</f>
+        <v/>
+      </c>
+      <c r="T11" s="6">
+        <f>IF(P11&gt;='Inputs'!$B$11,"LIQUIDATED",IF(P11&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(P11&gt;='Inputs'!$B$23,S11&lt;'Inputs'!$B$12),"WARNING",IF(AND(G11&gt;0,I11=0),"FAILED",IF(I11&lt;G11,"CONSTRAINED","SAFE")))))</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -2763,61 +3115,77 @@
         <f>'Price Projection'!B12</f>
         <v/>
       </c>
-      <c r="C12" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" s="11" t="n">
-        <v>74405.56200000001</v>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>7440.556200000001</v>
-      </c>
-      <c r="F12" s="11" t="n">
-        <v>81846.11820000001</v>
-      </c>
-      <c r="G12" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="H12" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="K12" s="11" t="n">
-        <v>42000</v>
-      </c>
-      <c r="L12" s="11" t="n">
-        <v>81846.11820000001</v>
-      </c>
-      <c r="M12" s="13" t="n">
-        <v>1.36410197</v>
-      </c>
-      <c r="N12" s="13" t="n">
-        <v>0.6358980299999999</v>
-      </c>
-      <c r="O12" s="11" t="n">
-        <v>38153.88179999999</v>
-      </c>
-      <c r="P12" s="12" t="n">
-        <v>0.6820509850000001</v>
-      </c>
-      <c r="Q12" s="11" t="n">
-        <v>58461.51300000001</v>
-      </c>
-      <c r="R12" s="11" t="n">
-        <v>54564.07880000001</v>
-      </c>
-      <c r="S12" s="12" t="n">
-        <v>0.09059868666666648</v>
-      </c>
-      <c r="T12" s="6" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
+      <c r="C12" s="13">
+        <f>'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="D12" s="11">
+        <f>L11</f>
+        <v/>
+      </c>
+      <c r="E12" s="11">
+        <f>D12*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F12" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D12+E12,D12)</f>
+        <v/>
+      </c>
+      <c r="G12" s="11">
+        <f>'Inputs'!$B$19</f>
+        <v/>
+      </c>
+      <c r="H12" s="11">
+        <f>MAX(0,MIN(C12*B12*'Inputs'!$B$20,C12*B12*'Inputs'!$B$11*(1-'Inputs'!$B$12))-F12)</f>
+        <v/>
+      </c>
+      <c r="I12" s="11">
+        <f>IF(IF(C12*B12=0,0,F12/(C12*B12))&gt;='Inputs'!$B$10,0,MIN(G12,H12))</f>
+        <v/>
+      </c>
+      <c r="J12" s="11">
+        <f>G12-I12</f>
+        <v/>
+      </c>
+      <c r="K12" s="11">
+        <f>K11+I12</f>
+        <v/>
+      </c>
+      <c r="L12" s="11">
+        <f>F12+I12</f>
+        <v/>
+      </c>
+      <c r="M12" s="13">
+        <f>L12/B12</f>
+        <v/>
+      </c>
+      <c r="N12" s="13">
+        <f>C12-M12</f>
+        <v/>
+      </c>
+      <c r="O12" s="11">
+        <f>C12*B12-L12</f>
+        <v/>
+      </c>
+      <c r="P12" s="12">
+        <f>IF(C12*B12=0,0,L12/(C12*B12))</f>
+        <v/>
+      </c>
+      <c r="Q12" s="11">
+        <f>IF(L12=0,0,L12/(C12*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="R12" s="11">
+        <f>IF(L12=0,0,L12/(C12*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="S12" s="12">
+        <f>IF(R12&lt;=0,0,1-R12/B12)</f>
+        <v/>
+      </c>
+      <c r="T12" s="6">
+        <f>IF(P12&gt;='Inputs'!$B$11,"LIQUIDATED",IF(P12&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(P12&gt;='Inputs'!$B$23,S12&lt;'Inputs'!$B$12),"WARNING",IF(AND(G12&gt;0,I12=0),"FAILED",IF(I12&lt;G12,"CONSTRAINED","SAFE")))))</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -2828,61 +3196,77 @@
         <f>'Price Projection'!B13</f>
         <v/>
       </c>
-      <c r="C13" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D13" s="11" t="n">
-        <v>81846.11820000001</v>
-      </c>
-      <c r="E13" s="11" t="n">
-        <v>8184.611820000002</v>
-      </c>
-      <c r="F13" s="11" t="n">
-        <v>90030.73002000002</v>
-      </c>
-      <c r="G13" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="H13" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="K13" s="11" t="n">
-        <v>42000</v>
-      </c>
-      <c r="L13" s="11" t="n">
-        <v>90030.73002000002</v>
-      </c>
-      <c r="M13" s="13" t="n">
-        <v>1.500512167</v>
-      </c>
-      <c r="N13" s="13" t="n">
-        <v>0.4994878329999997</v>
-      </c>
-      <c r="O13" s="11" t="n">
-        <v>29969.26997999998</v>
-      </c>
-      <c r="P13" s="12" t="n">
-        <v>0.7502560835000002</v>
-      </c>
-      <c r="Q13" s="11" t="n">
-        <v>64307.66430000002</v>
-      </c>
-      <c r="R13" s="11" t="n">
-        <v>60020.48668000001</v>
-      </c>
-      <c r="S13" s="12" t="n">
-        <v>-0.0003414446666667459</v>
-      </c>
-      <c r="T13" s="6" t="inlineStr">
-        <is>
-          <t>LIQUIDATED</t>
-        </is>
+      <c r="C13" s="13">
+        <f>'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="D13" s="11">
+        <f>L12</f>
+        <v/>
+      </c>
+      <c r="E13" s="11">
+        <f>D13*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F13" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D13+E13,D13)</f>
+        <v/>
+      </c>
+      <c r="G13" s="11">
+        <f>'Inputs'!$B$19</f>
+        <v/>
+      </c>
+      <c r="H13" s="11">
+        <f>MAX(0,MIN(C13*B13*'Inputs'!$B$20,C13*B13*'Inputs'!$B$11*(1-'Inputs'!$B$12))-F13)</f>
+        <v/>
+      </c>
+      <c r="I13" s="11">
+        <f>IF(IF(C13*B13=0,0,F13/(C13*B13))&gt;='Inputs'!$B$10,0,MIN(G13,H13))</f>
+        <v/>
+      </c>
+      <c r="J13" s="11">
+        <f>G13-I13</f>
+        <v/>
+      </c>
+      <c r="K13" s="11">
+        <f>K12+I13</f>
+        <v/>
+      </c>
+      <c r="L13" s="11">
+        <f>F13+I13</f>
+        <v/>
+      </c>
+      <c r="M13" s="13">
+        <f>L13/B13</f>
+        <v/>
+      </c>
+      <c r="N13" s="13">
+        <f>C13-M13</f>
+        <v/>
+      </c>
+      <c r="O13" s="11">
+        <f>C13*B13-L13</f>
+        <v/>
+      </c>
+      <c r="P13" s="12">
+        <f>IF(C13*B13=0,0,L13/(C13*B13))</f>
+        <v/>
+      </c>
+      <c r="Q13" s="11">
+        <f>IF(L13=0,0,L13/(C13*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="R13" s="11">
+        <f>IF(L13=0,0,L13/(C13*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="S13" s="12">
+        <f>IF(R13&lt;=0,0,1-R13/B13)</f>
+        <v/>
+      </c>
+      <c r="T13" s="6">
+        <f>IF(P13&gt;='Inputs'!$B$11,"LIQUIDATED",IF(P13&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(P13&gt;='Inputs'!$B$23,S13&lt;'Inputs'!$B$12),"WARNING",IF(AND(G13&gt;0,I13=0),"FAILED",IF(I13&lt;G13,"CONSTRAINED","SAFE")))))</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -2893,61 +3277,77 @@
         <f>'Price Projection'!B14</f>
         <v/>
       </c>
-      <c r="C14" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D14" s="11" t="n">
-        <v>90030.73002000002</v>
-      </c>
-      <c r="E14" s="11" t="n">
-        <v>9003.073002000003</v>
-      </c>
-      <c r="F14" s="11" t="n">
-        <v>99033.80302200002</v>
-      </c>
-      <c r="G14" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="H14" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="K14" s="11" t="n">
-        <v>42000</v>
-      </c>
-      <c r="L14" s="11" t="n">
-        <v>99033.80302200002</v>
-      </c>
-      <c r="M14" s="13" t="n">
-        <v>1.6505633837</v>
-      </c>
-      <c r="N14" s="13" t="n">
-        <v>0.3494366162999996</v>
-      </c>
-      <c r="O14" s="11" t="n">
-        <v>20966.19697799998</v>
-      </c>
-      <c r="P14" s="12" t="n">
-        <v>0.8252816918500002</v>
-      </c>
-      <c r="Q14" s="11" t="n">
-        <v>70738.43073000002</v>
-      </c>
-      <c r="R14" s="11" t="n">
-        <v>66022.53534800002</v>
-      </c>
-      <c r="S14" s="12" t="n">
-        <v>-0.1003755891333336</v>
-      </c>
-      <c r="T14" s="6" t="inlineStr">
-        <is>
-          <t>LIQUIDATED</t>
-        </is>
+      <c r="C14" s="13">
+        <f>'Inputs'!$B$7</f>
+        <v/>
+      </c>
+      <c r="D14" s="11">
+        <f>L13</f>
+        <v/>
+      </c>
+      <c r="E14" s="11">
+        <f>D14*'Inputs'!$B$8</f>
+        <v/>
+      </c>
+      <c r="F14" s="11">
+        <f>IF('Inputs'!$B$9="capitalized",D14+E14,D14)</f>
+        <v/>
+      </c>
+      <c r="G14" s="11">
+        <f>'Inputs'!$B$19</f>
+        <v/>
+      </c>
+      <c r="H14" s="11">
+        <f>MAX(0,MIN(C14*B14*'Inputs'!$B$20,C14*B14*'Inputs'!$B$11*(1-'Inputs'!$B$12))-F14)</f>
+        <v/>
+      </c>
+      <c r="I14" s="11">
+        <f>IF(IF(C14*B14=0,0,F14/(C14*B14))&gt;='Inputs'!$B$10,0,MIN(G14,H14))</f>
+        <v/>
+      </c>
+      <c r="J14" s="11">
+        <f>G14-I14</f>
+        <v/>
+      </c>
+      <c r="K14" s="11">
+        <f>K13+I14</f>
+        <v/>
+      </c>
+      <c r="L14" s="11">
+        <f>F14+I14</f>
+        <v/>
+      </c>
+      <c r="M14" s="13">
+        <f>L14/B14</f>
+        <v/>
+      </c>
+      <c r="N14" s="13">
+        <f>C14-M14</f>
+        <v/>
+      </c>
+      <c r="O14" s="11">
+        <f>C14*B14-L14</f>
+        <v/>
+      </c>
+      <c r="P14" s="12">
+        <f>IF(C14*B14=0,0,L14/(C14*B14))</f>
+        <v/>
+      </c>
+      <c r="Q14" s="11">
+        <f>IF(L14=0,0,L14/(C14*'Inputs'!$B$10))</f>
+        <v/>
+      </c>
+      <c r="R14" s="11">
+        <f>IF(L14=0,0,L14/(C14*'Inputs'!$B$11))</f>
+        <v/>
+      </c>
+      <c r="S14" s="12">
+        <f>IF(R14&lt;=0,0,1-R14/B14)</f>
+        <v/>
+      </c>
+      <c r="T14" s="6">
+        <f>IF(P14&gt;='Inputs'!$B$11,"LIQUIDATED",IF(P14&gt;='Inputs'!$B$10,"MARGIN CALL",IF(OR(P14&gt;='Inputs'!$B$23,S14&lt;'Inputs'!$B$12),"WARNING",IF(AND(G14&gt;0,I14=0),"FAILED",IF(I14&lt;G14,"CONSTRAINED","SAFE")))))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -2968,7 +3368,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -3010,8 +3410,9 @@
           <t>Accumulation max effective LTV</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0.6484356150250001</v>
+      <c r="B5" s="12">
+        <f>MAX('Accumulation Engine'!Q4:Q14)</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -3020,8 +3421,9 @@
           <t>Accumulation min drop-to-liquidation</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
-        <v>0.1354191799666664</v>
+      <c r="B6" s="12">
+        <f>MIN('Accumulation Engine'!U4:U14)</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -3030,8 +3432,9 @@
           <t>Accumulation first non-safe year</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
-        <v>5</v>
+      <c r="B7" s="6">
+        <f>IF(COUNTIF('Accumulation Engine'!$V$4:$V$14,"&lt;&gt;SAFE")=0,"None",INDEX('Accumulation Engine'!$A$4:$A$14,AGGREGATE(15,6,(ROW('Accumulation Engine'!$V$4:$V$14)-ROW('Accumulation Engine'!$V$4)+1)/('Accumulation Engine'!$V$4:$V$14&lt;&gt;"SAFE"),1)))</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -3040,10 +3443,9 @@
           <t>Accumulation liquidation year</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+      <c r="B8" s="6">
+        <f>IFERROR(INDEX('Accumulation Engine'!$A$4:$A$14,MATCH("LIQUIDATED",'Accumulation Engine'!$V$4:$V$14,0)),"None")</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -3052,8 +3454,9 @@
           <t>Accumulation total interest accrued</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n">
-        <v>63749.69840400001</v>
+      <c r="B9" s="11">
+        <f>SUM('Accumulation Engine'!E4:E14)</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -3062,8 +3465,9 @@
           <t>Accumulation total new borrowing</t>
         </is>
       </c>
-      <c r="B10" s="11" t="n">
-        <v>40000</v>
+      <c r="B10" s="11">
+        <f>SUM('Accumulation Engine'!H4:H14)</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -3072,8 +3476,9 @@
           <t>Accumulation ending net BTC</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n">
-        <v>0.9375050265999993</v>
+      <c r="B11" s="13">
+        <f>'Accumulation Engine'!N14</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -3082,8 +3487,9 @@
           <t>Accumulation BTC outperformance vs passive</t>
         </is>
       </c>
-      <c r="B12" s="13" t="n">
-        <v>-1.062494973400001</v>
+      <c r="B12" s="13">
+        <f>'Accumulation Engine'!N14-'Inputs'!$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -3099,8 +3505,9 @@
           <t>Income max effective LTV</t>
         </is>
       </c>
-      <c r="B14" s="12" t="n">
-        <v>0.8252816918500002</v>
+      <c r="B14" s="12">
+        <f>MAX('Income Engine'!P4:P14)</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -3109,8 +3516,9 @@
           <t>Income min drop-to-liquidation</t>
         </is>
       </c>
-      <c r="B15" s="12" t="n">
-        <v>-0.1003755891333336</v>
+      <c r="B15" s="12">
+        <f>MIN('Income Engine'!S4:S14)</f>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -3119,8 +3527,9 @@
           <t>Income first constrained year</t>
         </is>
       </c>
-      <c r="B16" s="6" t="n">
-        <v>1</v>
+      <c r="B16" s="6">
+        <f>IFERROR(INDEX('Income Engine'!$A$4:$A$14,MATCH("CONSTRAINED",'Income Engine'!$T$4:$T$14,0)),"None")</f>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -3129,8 +3538,9 @@
           <t>Income liquidation year</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n">
-        <v>9</v>
+      <c r="B17" s="6">
+        <f>IFERROR(INDEX('Income Engine'!$A$4:$A$14,MATCH("LIQUIDATED",'Income Engine'!$T$4:$T$14,0)),"None")</f>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -3139,8 +3549,9 @@
           <t>Income total interest accrued</t>
         </is>
       </c>
-      <c r="B18" s="11" t="n">
-        <v>57033.80302200001</v>
+      <c r="B18" s="11">
+        <f>SUM('Income Engine'!E4:E14)</f>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -3149,8 +3560,9 @@
           <t>Income total funded</t>
         </is>
       </c>
-      <c r="B19" s="11" t="n">
-        <v>42000</v>
+      <c r="B19" s="11">
+        <f>SUM('Income Engine'!I4:I14)</f>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -3159,8 +3571,9 @@
           <t>Income total shortfall</t>
         </is>
       </c>
-      <c r="B20" s="11" t="n">
-        <v>458000</v>
+      <c r="B20" s="11">
+        <f>SUM('Income Engine'!J4:J14)</f>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -3176,8 +3589,9 @@
           <t>Passive BTC held</t>
         </is>
       </c>
-      <c r="B22" s="13" t="n">
-        <v>2</v>
+      <c r="B22" s="13">
+        <f>'Inputs'!$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -3186,8 +3600,9 @@
           <t>Passive ending value</t>
         </is>
       </c>
-      <c r="B23" s="11" t="n">
-        <v>120000</v>
+      <c r="B23" s="11">
+        <f>'Inputs'!$B$7*'Price Projection'!B14</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -3211,7 +3626,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -3246,8 +3661,9 @@
           <t>Passive starting BTC</t>
         </is>
       </c>
-      <c r="B4" s="13" t="n">
-        <v>2</v>
+      <c r="B4" s="13">
+        <f>'Inputs'!$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -3256,8 +3672,9 @@
           <t>Passive ending BTC</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n">
-        <v>2</v>
+      <c r="B5" s="13">
+        <f>'Inputs'!$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -3266,8 +3683,9 @@
           <t>Passive ending value</t>
         </is>
       </c>
-      <c r="B6" s="11" t="n">
-        <v>120000</v>
+      <c r="B6" s="11">
+        <f>'Inputs'!$B$7*'Price Projection'!B14</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -3276,8 +3694,9 @@
           <t>Accumulation setup gross BTC</t>
         </is>
       </c>
-      <c r="B7" s="13" t="n">
-        <v>2.666666666666667</v>
+      <c r="B7" s="13">
+        <f>'Accumulation Engine'!J4</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -3286,8 +3705,9 @@
           <t>Accumulation ending gross BTC</t>
         </is>
       </c>
-      <c r="B8" s="13" t="n">
-        <v>2.666666666666667</v>
+      <c r="B8" s="13">
+        <f>'Accumulation Engine'!J14</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -3296,8 +3716,9 @@
           <t>Accumulation ending debt</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n">
-        <v>103749.698404</v>
+      <c r="B9" s="11">
+        <f>'Accumulation Engine'!K14</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -3306,8 +3727,9 @@
           <t>Accumulation ending net BTC</t>
         </is>
       </c>
-      <c r="B10" s="13" t="n">
-        <v>0.9375050265999993</v>
+      <c r="B10" s="13">
+        <f>'Accumulation Engine'!N14</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -3316,8 +3738,9 @@
           <t>Accumulation ending LTV</t>
         </is>
       </c>
-      <c r="B11" s="12" t="n">
-        <v>0.6484356150250001</v>
+      <c r="B11" s="12">
+        <f>'Accumulation Engine'!Q14</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -3326,10 +3749,9 @@
           <t>Accumulation status</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
+      <c r="B12" s="6">
+        <f>'Accumulation Engine'!V14</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -3338,8 +3760,9 @@
           <t>Income selected draw year 1</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n">
-        <v>50000</v>
+      <c r="B13" s="11">
+        <f>'Inputs'!$B$19</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -3348,8 +3771,9 @@
           <t>Income funded year 1</t>
         </is>
       </c>
-      <c r="B14" s="11" t="n">
-        <v>42000</v>
+      <c r="B14" s="11">
+        <f>'Income Engine'!I5</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -3358,8 +3782,9 @@
           <t>Income shortfall year 1</t>
         </is>
       </c>
-      <c r="B15" s="11" t="n">
-        <v>8000</v>
+      <c r="B15" s="11">
+        <f>'Income Engine'!J5</f>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -3368,8 +3793,9 @@
           <t>Income ending debt</t>
         </is>
       </c>
-      <c r="B16" s="11" t="n">
-        <v>99033.80302200002</v>
+      <c r="B16" s="11">
+        <f>'Income Engine'!L14</f>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -3378,8 +3804,9 @@
           <t>Income ending net BTC</t>
         </is>
       </c>
-      <c r="B17" s="13" t="n">
-        <v>0.3494366162999996</v>
+      <c r="B17" s="13">
+        <f>'Income Engine'!N14</f>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -3388,10 +3815,9 @@
           <t>Income status</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>LIQUIDATED</t>
-        </is>
+      <c r="B18" s="6">
+        <f>'Income Engine'!T14</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>